<commit_message>
data(hsk6): Bài 29 例句 cá nhân hoá + 生词拓展 có nghĩa
- 49 例句 thay bằng câu cá nhân hoá (tự học/luyện thi HSK6, làm việc TQ,
  dạy HSK1-3), bỏ câu trùng slide.
- 生词拓展 Bài 29: 9 nhóm họ chữ + nghĩa Việt từng từ con.
- Regenerate tu-vung.{md,html}.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/raw/Từ vựng.xlsx
+++ b/raw/Từ vựng.xlsx
@@ -71007,1670 +71007,1670 @@
       </c>
     </row>
     <row r="3026">
-      <c r="A3026" t="inlineStr">
+      <c r="A3026" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3026" t="inlineStr">
+      <c r="B3026" s="0" t="inlineStr">
         <is>
           <t>难堪</t>
         </is>
       </c>
-      <c r="C3026" t="inlineStr">
+      <c r="C3026" s="0" t="inlineStr">
         <is>
           <t>nánkān</t>
         </is>
       </c>
-      <c r="D3026" t="inlineStr">
+      <c r="D3026" s="0" t="inlineStr">
         <is>
           <t>感到很不好意思，很尴尬，下不来台</t>
         </is>
       </c>
-      <c r="E3026" t="inlineStr">
+      <c r="E3026" s="0" t="inlineStr">
         <is>
           <t>khó xử, bẽ bàng, ngượng</t>
         </is>
       </c>
-      <c r="F3026" t="inlineStr">
-        <is>
-          <t>这件事情让他感到很难堪，脸都涨红了。</t>
-        </is>
-      </c>
-      <c r="G3026" t="inlineStr"/>
-      <c r="H3026" t="inlineStr"/>
+      <c r="F3026" s="0" t="inlineStr">
+        <is>
+          <t>上课时被学生问到一个我也不太确定的语法，我一时有点难堪。</t>
+        </is>
+      </c>
+      <c r="G3026" s="0" t="inlineStr"/>
+      <c r="H3026" s="0" t="inlineStr"/>
     </row>
     <row r="3027">
-      <c r="A3027" t="inlineStr">
+      <c r="A3027" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3027" t="inlineStr">
+      <c r="B3027" s="0" t="inlineStr">
         <is>
           <t>岂有此理</t>
         </is>
       </c>
-      <c r="C3027" t="inlineStr">
+      <c r="C3027" s="0" t="inlineStr">
         <is>
           <t>qǐyǒucǐlǐ</t>
         </is>
       </c>
-      <c r="D3027" t="inlineStr">
+      <c r="D3027" s="0" t="inlineStr">
         <is>
           <t>哪有这样的道理；表示对不合理的事很生气</t>
         </is>
       </c>
-      <c r="E3027" t="inlineStr">
+      <c r="E3027" s="0" t="inlineStr">
         <is>
           <t>thật vô lý, làm gì có cái lý đó</t>
         </is>
       </c>
-      <c r="F3027" t="inlineStr">
-        <is>
-          <t>大家好心问你，你倒说别人多管闲事，真是岂有此理！</t>
-        </is>
-      </c>
-      <c r="G3027" t="inlineStr"/>
-      <c r="H3027" t="inlineStr"/>
+      <c r="F3027" s="0" t="inlineStr">
+        <is>
+          <t>我熬夜背了那么多生词，考试居然一个都没考到，真是岂有此理！</t>
+        </is>
+      </c>
+      <c r="G3027" s="0" t="inlineStr"/>
+      <c r="H3027" s="0" t="inlineStr"/>
     </row>
     <row r="3028">
-      <c r="A3028" t="inlineStr">
+      <c r="A3028" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3028" t="inlineStr">
+      <c r="B3028" s="0" t="inlineStr">
         <is>
           <t>庸俗</t>
         </is>
       </c>
-      <c r="C3028" t="inlineStr">
+      <c r="C3028" s="0" t="inlineStr">
         <is>
           <t>yōngsú</t>
         </is>
       </c>
-      <c r="D3028" t="inlineStr">
+      <c r="D3028" s="0" t="inlineStr">
         <is>
           <t>不高雅，低级，没有品味</t>
         </is>
       </c>
-      <c r="E3028" t="inlineStr">
+      <c r="E3028" s="0" t="inlineStr">
         <is>
           <t>tầm thường, dung tục</t>
         </is>
       </c>
-      <c r="F3028" t="inlineStr">
-        <is>
-          <t>这歌曲的歌词太庸俗了。</t>
-        </is>
-      </c>
-      <c r="G3028" t="inlineStr"/>
-      <c r="H3028" t="inlineStr"/>
+      <c r="F3028" s="0" t="inlineStr">
+        <is>
+          <t>我不太喜欢那种只谈钱、谈名牌的庸俗话题。</t>
+        </is>
+      </c>
+      <c r="G3028" s="0" t="inlineStr"/>
+      <c r="H3028" s="0" t="inlineStr"/>
     </row>
     <row r="3029">
-      <c r="A3029" t="inlineStr">
+      <c r="A3029" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3029" t="inlineStr">
+      <c r="B3029" s="0" t="inlineStr">
         <is>
           <t>档次</t>
         </is>
       </c>
-      <c r="C3029" t="inlineStr">
+      <c r="C3029" s="0" t="inlineStr">
         <is>
           <t>dàngcì</t>
         </is>
       </c>
-      <c r="D3029" t="inlineStr">
+      <c r="D3029" s="0" t="inlineStr">
         <is>
           <t>按质量或水平分出的高低等级</t>
         </is>
       </c>
-      <c r="E3029" t="inlineStr">
+      <c r="E3029" s="0" t="inlineStr">
         <is>
           <t>đẳng cấp, thứ hạng</t>
         </is>
       </c>
-      <c r="F3029" t="inlineStr">
-        <is>
-          <t>业主消费档次和消费要求不一样，真让我为难。</t>
-        </is>
-      </c>
-      <c r="G3029" t="inlineStr"/>
-      <c r="H3029" t="inlineStr"/>
+      <c r="F3029" s="0" t="inlineStr">
+        <is>
+          <t>这家咖啡馆虽然不大，但装修和服务都挺有档次的。</t>
+        </is>
+      </c>
+      <c r="G3029" s="0" t="inlineStr"/>
+      <c r="H3029" s="0" t="inlineStr"/>
     </row>
     <row r="3030">
-      <c r="A3030" t="inlineStr">
+      <c r="A3030" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3030" t="inlineStr">
+      <c r="B3030" s="0" t="inlineStr">
         <is>
           <t>诸位</t>
         </is>
       </c>
-      <c r="C3030" t="inlineStr">
+      <c r="C3030" s="0" t="inlineStr">
         <is>
           <t>zhūwèi</t>
         </is>
       </c>
-      <c r="D3030" t="inlineStr">
+      <c r="D3030" s="0" t="inlineStr">
         <is>
           <t>对很多人的尊称，各位</t>
         </is>
       </c>
-      <c r="E3030" t="inlineStr">
+      <c r="E3030" s="0" t="inlineStr">
         <is>
           <t>chư vị, các vị (các anh chị)</t>
         </is>
       </c>
-      <c r="F3030" t="inlineStr">
-        <is>
-          <t>以上是我对该书的一点见解，仅供诸位参考。</t>
-        </is>
-      </c>
-      <c r="G3030" t="inlineStr"/>
-      <c r="H3030" t="inlineStr"/>
+      <c r="F3030" s="0" t="inlineStr">
+        <is>
+          <t>上课第一天我常对学生说：“诸位，学中文最重要的就是坚持。”</t>
+        </is>
+      </c>
+      <c r="G3030" s="0" t="inlineStr"/>
+      <c r="H3030" s="0" t="inlineStr"/>
     </row>
     <row r="3031">
-      <c r="A3031" t="inlineStr">
+      <c r="A3031" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3031" t="inlineStr">
+      <c r="B3031" s="0" t="inlineStr">
         <is>
           <t>预先</t>
         </is>
       </c>
-      <c r="C3031" t="inlineStr">
+      <c r="C3031" s="0" t="inlineStr">
         <is>
           <t>yùxiān</t>
         </is>
       </c>
-      <c r="D3031" t="inlineStr">
+      <c r="D3031" s="0" t="inlineStr">
         <is>
           <t>在事情发生之前就先做某事</t>
         </is>
       </c>
-      <c r="E3031" t="inlineStr">
+      <c r="E3031" s="0" t="inlineStr">
         <is>
           <t>trước, từ trước</t>
         </is>
       </c>
-      <c r="F3031" t="inlineStr">
-        <is>
-          <t>洪水到来之前，我们得到了有关部门的预先通知。</t>
-        </is>
-      </c>
-      <c r="G3031" t="inlineStr"/>
-      <c r="H3031" t="inlineStr"/>
+      <c r="F3031" s="0" t="inlineStr">
+        <is>
+          <t>明天要跟中国同事开会，我得预先把要说的话准备好。</t>
+        </is>
+      </c>
+      <c r="G3031" s="0" t="inlineStr"/>
+      <c r="H3031" s="0" t="inlineStr"/>
     </row>
     <row r="3032">
-      <c r="A3032" t="inlineStr">
+      <c r="A3032" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3032" t="inlineStr">
+      <c r="B3032" s="0" t="inlineStr">
         <is>
           <t>直觉</t>
         </is>
       </c>
-      <c r="C3032" t="inlineStr">
+      <c r="C3032" s="0" t="inlineStr">
         <is>
           <t>zhíjué</t>
         </is>
       </c>
-      <c r="D3032" t="inlineStr">
+      <c r="D3032" s="0" t="inlineStr">
         <is>
           <t>不用思考就直接感觉到的判断</t>
         </is>
       </c>
-      <c r="E3032" t="inlineStr">
+      <c r="E3032" s="0" t="inlineStr">
         <is>
           <t>trực giác</t>
         </is>
       </c>
-      <c r="F3032" t="inlineStr">
-        <is>
-          <t>其实他并不确定是哪条路，但直觉告诉他，要左拐。</t>
-        </is>
-      </c>
-      <c r="G3032" t="inlineStr"/>
-      <c r="H3032" t="inlineStr"/>
+      <c r="F3032" s="0" t="inlineStr">
+        <is>
+          <t>做HSK阅读题时，有时候我会先凭直觉选一个答案，再回头检查。</t>
+        </is>
+      </c>
+      <c r="G3032" s="0" t="inlineStr"/>
+      <c r="H3032" s="0" t="inlineStr"/>
     </row>
     <row r="3033">
-      <c r="A3033" t="inlineStr">
+      <c r="A3033" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3033" t="inlineStr">
+      <c r="B3033" s="0" t="inlineStr">
         <is>
           <t>座右铭</t>
         </is>
       </c>
-      <c r="C3033" t="inlineStr">
+      <c r="C3033" s="0" t="inlineStr">
         <is>
           <t>zuòyòumíng</t>
         </is>
       </c>
-      <c r="D3033" t="inlineStr">
+      <c r="D3033" s="0" t="inlineStr">
         <is>
           <t>用来提醒、勉励自己的一句话</t>
         </is>
       </c>
-      <c r="E3033" t="inlineStr">
+      <c r="E3033" s="0" t="inlineStr">
         <is>
           <t>châm ngôn (tự nhắc mình)</t>
         </is>
       </c>
-      <c r="F3033" t="inlineStr">
-        <is>
-          <t>人人为我，我为人人，这是我们的座右铭。</t>
-        </is>
-      </c>
-      <c r="G3033" t="inlineStr"/>
-      <c r="H3033" t="inlineStr"/>
+      <c r="F3033" s="0" t="inlineStr">
+        <is>
+          <t>“坚持就是胜利”是我备考路上的座右铭。</t>
+        </is>
+      </c>
+      <c r="G3033" s="0" t="inlineStr"/>
+      <c r="H3033" s="0" t="inlineStr"/>
     </row>
     <row r="3034">
-      <c r="A3034" t="inlineStr">
+      <c r="A3034" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3034" t="inlineStr">
+      <c r="B3034" s="0" t="inlineStr">
         <is>
           <t>通用</t>
         </is>
       </c>
-      <c r="C3034" t="inlineStr">
+      <c r="C3034" s="0" t="inlineStr">
         <is>
           <t>tōngyòng</t>
         </is>
       </c>
-      <c r="D3034" t="inlineStr">
+      <c r="D3034" s="0" t="inlineStr">
         <is>
           <t>大家都可以用，普遍使用</t>
         </is>
       </c>
-      <c r="E3034" t="inlineStr">
+      <c r="E3034" s="0" t="inlineStr">
         <is>
           <t>dùng chung, thông dụng</t>
         </is>
       </c>
-      <c r="F3034" t="inlineStr">
-        <is>
-          <t>微笑是一种国际通用的语言。</t>
-        </is>
-      </c>
-      <c r="G3034" t="inlineStr"/>
-      <c r="H3034" t="inlineStr"/>
+      <c r="F3034" s="0" t="inlineStr">
+        <is>
+          <t>微笑和礼貌几乎在哪个国家都是通用的。</t>
+        </is>
+      </c>
+      <c r="G3034" s="0" t="inlineStr"/>
+      <c r="H3034" s="0" t="inlineStr"/>
     </row>
     <row r="3035">
-      <c r="A3035" t="inlineStr">
+      <c r="A3035" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3035" t="inlineStr">
+      <c r="B3035" s="0" t="inlineStr">
         <is>
           <t>调节</t>
         </is>
       </c>
-      <c r="C3035" t="inlineStr">
+      <c r="C3035" s="0" t="inlineStr">
         <is>
           <t>tiáojié</t>
         </is>
       </c>
-      <c r="D3035" t="inlineStr">
+      <c r="D3035" s="0" t="inlineStr">
         <is>
           <t>调整，使更合适、更协调</t>
         </is>
       </c>
-      <c r="E3035" t="inlineStr">
+      <c r="E3035" s="0" t="inlineStr">
         <is>
           <t>điều tiết, điều hòa</t>
         </is>
       </c>
-      <c r="F3035" t="inlineStr">
-        <is>
-          <t>老师为我调节了与同学之间的矛盾。</t>
-        </is>
-      </c>
-      <c r="G3035" t="inlineStr"/>
-      <c r="H3035" t="inlineStr"/>
+      <c r="F3035" s="0" t="inlineStr">
+        <is>
+          <t>工作压力大的时候，我会用跑步来调节自己的情绪。</t>
+        </is>
+      </c>
+      <c r="G3035" s="0" t="inlineStr"/>
+      <c r="H3035" s="0" t="inlineStr"/>
     </row>
     <row r="3036">
-      <c r="A3036" t="inlineStr">
+      <c r="A3036" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3036" t="inlineStr">
+      <c r="B3036" s="0" t="inlineStr">
         <is>
           <t>循环</t>
         </is>
       </c>
-      <c r="C3036" t="inlineStr">
+      <c r="C3036" s="0" t="inlineStr">
         <is>
           <t>xúnhuán</t>
         </is>
       </c>
-      <c r="D3036" t="inlineStr">
+      <c r="D3036" s="0" t="inlineStr">
         <is>
           <t>按顺序重复地运行一圈又一圈</t>
         </is>
       </c>
-      <c r="E3036" t="inlineStr">
+      <c r="E3036" s="0" t="inlineStr">
         <is>
           <t>tuần hoàn</t>
         </is>
       </c>
-      <c r="F3036" t="inlineStr">
-        <is>
-          <t>由于药物的作用，血液循环加快了。</t>
-        </is>
-      </c>
-      <c r="G3036" t="inlineStr"/>
-      <c r="H3036" t="inlineStr"/>
+      <c r="F3036" s="0" t="inlineStr">
+        <is>
+          <t>早睡早起形成良性循环，我白天学习的效率就高多了。</t>
+        </is>
+      </c>
+      <c r="G3036" s="0" t="inlineStr"/>
+      <c r="H3036" s="0" t="inlineStr"/>
     </row>
     <row r="3037">
-      <c r="A3037" t="inlineStr">
+      <c r="A3037" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3037" t="inlineStr">
+      <c r="B3037" s="0" t="inlineStr">
         <is>
           <t>收缩</t>
         </is>
       </c>
-      <c r="C3037" t="inlineStr">
+      <c r="C3037" s="0" t="inlineStr">
         <is>
           <t>shōusuō</t>
         </is>
       </c>
-      <c r="D3037" t="inlineStr">
+      <c r="D3037" s="0" t="inlineStr">
         <is>
           <t>由大变小、往里缩</t>
         </is>
       </c>
-      <c r="E3037" t="inlineStr">
+      <c r="E3037" s="0" t="inlineStr">
         <is>
           <t>co lại, thu nhỏ</t>
         </is>
       </c>
-      <c r="F3037" t="inlineStr">
-        <is>
-          <t>含羞草一受刺激，叶子就收缩起来。</t>
-        </is>
-      </c>
-      <c r="G3037" t="inlineStr"/>
-      <c r="H3037" t="inlineStr"/>
+      <c r="F3037" s="0" t="inlineStr">
+        <is>
+          <t>运动完一定要拉伸，不然肌肉一直收缩，第二天会很酸。</t>
+        </is>
+      </c>
+      <c r="G3037" s="0" t="inlineStr"/>
+      <c r="H3037" s="0" t="inlineStr"/>
     </row>
     <row r="3038">
-      <c r="A3038" t="inlineStr">
+      <c r="A3038" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3038" t="inlineStr">
+      <c r="B3038" s="0" t="inlineStr">
         <is>
           <t>氧气</t>
         </is>
       </c>
-      <c r="C3038" t="inlineStr">
+      <c r="C3038" s="0" t="inlineStr">
         <is>
           <t>yǎngqì</t>
         </is>
       </c>
-      <c r="D3038" t="inlineStr">
+      <c r="D3038" s="0" t="inlineStr">
         <is>
           <t>空气里让人呼吸、能助燃的气体</t>
         </is>
       </c>
-      <c r="E3038" t="inlineStr">
+      <c r="E3038" s="0" t="inlineStr">
         <is>
           <t>khí oxy</t>
         </is>
       </c>
-      <c r="F3038" t="inlineStr">
-        <is>
-          <t>因为有氧气，所以地球上才有生命。</t>
-        </is>
-      </c>
-      <c r="G3038" t="inlineStr"/>
-      <c r="H3038" t="inlineStr"/>
+      <c r="F3038" s="0" t="inlineStr">
+        <is>
+          <t>房间闷的时候我会开窗，让新鲜氧气进来，脑子也清醒些。</t>
+        </is>
+      </c>
+      <c r="G3038" s="0" t="inlineStr"/>
+      <c r="H3038" s="0" t="inlineStr"/>
     </row>
     <row r="3039">
-      <c r="A3039" t="inlineStr">
+      <c r="A3039" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3039" t="inlineStr">
+      <c r="B3039" s="0" t="inlineStr">
         <is>
           <t>斟酌</t>
         </is>
       </c>
-      <c r="C3039" t="inlineStr">
+      <c r="C3039" s="0" t="inlineStr">
         <is>
           <t>zhēnzhuó</t>
         </is>
       </c>
-      <c r="D3039" t="inlineStr">
+      <c r="D3039" s="0" t="inlineStr">
         <is>
           <t>反复考虑，仔细掂量该怎么做</t>
         </is>
       </c>
-      <c r="E3039" t="inlineStr">
+      <c r="E3039" s="0" t="inlineStr">
         <is>
           <t>cân nhắc, đắn đo</t>
         </is>
       </c>
-      <c r="F3039" t="inlineStr">
-        <is>
-          <t>事情比较复杂，怎么处理，还得斟酌一下。</t>
-        </is>
-      </c>
-      <c r="G3039" t="inlineStr"/>
-      <c r="H3039" t="inlineStr"/>
+      <c r="F3039" s="0" t="inlineStr">
+        <is>
+          <t>给学生写评语时，我会反复斟酌用词，怕伤到他们的自信。</t>
+        </is>
+      </c>
+      <c r="G3039" s="0" t="inlineStr"/>
+      <c r="H3039" s="0" t="inlineStr"/>
     </row>
     <row r="3040">
-      <c r="A3040" t="inlineStr">
+      <c r="A3040" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3040" t="inlineStr">
+      <c r="B3040" s="0" t="inlineStr">
         <is>
           <t>虚伪</t>
         </is>
       </c>
-      <c r="C3040" t="inlineStr">
+      <c r="C3040" s="0" t="inlineStr">
         <is>
           <t>xūwěi</t>
         </is>
       </c>
-      <c r="D3040" t="inlineStr">
+      <c r="D3040" s="0" t="inlineStr">
         <is>
           <t>不真实，假装的，表里不一</t>
         </is>
       </c>
-      <c r="E3040" t="inlineStr">
+      <c r="E3040" s="0" t="inlineStr">
         <is>
           <t>giả dối, đạo đức giả</t>
         </is>
       </c>
-      <c r="F3040" t="inlineStr">
-        <is>
-          <t>法官揭露了这个坏蛋虚伪的面目。</t>
-        </is>
-      </c>
-      <c r="G3040" t="inlineStr"/>
-      <c r="H3040" t="inlineStr"/>
+      <c r="F3040" s="0" t="inlineStr">
+        <is>
+          <t>我不太会应付那种表面客气、其实很虚伪的人。</t>
+        </is>
+      </c>
+      <c r="G3040" s="0" t="inlineStr"/>
+      <c r="H3040" s="0" t="inlineStr"/>
     </row>
     <row r="3041">
-      <c r="A3041" t="inlineStr">
+      <c r="A3041" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3041" t="inlineStr">
+      <c r="B3041" s="0" t="inlineStr">
         <is>
           <t>违背</t>
         </is>
       </c>
-      <c r="C3041" t="inlineStr">
+      <c r="C3041" s="0" t="inlineStr">
         <is>
           <t>wéibèi</t>
         </is>
       </c>
-      <c r="D3041" t="inlineStr">
+      <c r="D3041" s="0" t="inlineStr">
         <is>
           <t>不遵守，跟…相反</t>
         </is>
       </c>
-      <c r="E3041" t="inlineStr">
+      <c r="E3041" s="0" t="inlineStr">
         <is>
           <t>làm trái, đi ngược lại</t>
         </is>
       </c>
-      <c r="F3041" t="inlineStr">
-        <is>
-          <t>哥哥违背了爸爸的意愿当了一名医生。</t>
-        </is>
-      </c>
-      <c r="G3041" t="inlineStr"/>
-      <c r="H3041" t="inlineStr"/>
+      <c r="F3041" s="0" t="inlineStr">
+        <is>
+          <t>为了赶进度而违背学习规律，结果反而记不牢。</t>
+        </is>
+      </c>
+      <c r="G3041" s="0" t="inlineStr"/>
+      <c r="H3041" s="0" t="inlineStr"/>
     </row>
     <row r="3042">
-      <c r="A3042" t="inlineStr">
+      <c r="A3042" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3042" t="inlineStr">
+      <c r="B3042" s="0" t="inlineStr">
         <is>
           <t>回避</t>
         </is>
       </c>
-      <c r="C3042" t="inlineStr">
+      <c r="C3042" s="0" t="inlineStr">
         <is>
           <t>huíbì</t>
         </is>
       </c>
-      <c r="D3042" t="inlineStr">
+      <c r="D3042" s="0" t="inlineStr">
         <is>
           <t>有意躲开，不正面面对</t>
         </is>
       </c>
-      <c r="E3042" t="inlineStr">
+      <c r="E3042" s="0" t="inlineStr">
         <is>
           <t>né tránh</t>
         </is>
       </c>
-      <c r="F3042" t="inlineStr">
-        <is>
-          <t>不知为什么，他总是回避这个问题。</t>
-        </is>
-      </c>
-      <c r="G3042" t="inlineStr"/>
-      <c r="H3042" t="inlineStr"/>
+      <c r="F3042" s="0" t="inlineStr">
+        <is>
+          <t>遇到不会的语法，我不想回避，而是当场就查清楚。</t>
+        </is>
+      </c>
+      <c r="G3042" s="0" t="inlineStr"/>
+      <c r="H3042" s="0" t="inlineStr"/>
     </row>
     <row r="3043">
-      <c r="A3043" t="inlineStr">
+      <c r="A3043" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3043" t="inlineStr">
+      <c r="B3043" s="0" t="inlineStr">
         <is>
           <t>岔</t>
         </is>
       </c>
-      <c r="C3043" t="inlineStr">
+      <c r="C3043" s="0" t="inlineStr">
         <is>
           <t>chà</t>
         </is>
       </c>
-      <c r="D3043" t="inlineStr">
+      <c r="D3043" s="0" t="inlineStr">
         <is>
           <t>把话题引到别的方向</t>
         </is>
       </c>
-      <c r="E3043" t="inlineStr">
+      <c r="E3043" s="0" t="inlineStr">
         <is>
           <t>lái (chủ đề) sang chỗ khác</t>
         </is>
       </c>
-      <c r="F3043" t="inlineStr">
-        <is>
-          <t>他设法把讨论内容从钱的话题上岔开了。</t>
-        </is>
-      </c>
-      <c r="G3043" t="inlineStr"/>
-      <c r="H3043" t="inlineStr"/>
+      <c r="F3043" s="0" t="inlineStr">
+        <is>
+          <t>每次别人问我工资多少，我都赶紧把话题岔开。</t>
+        </is>
+      </c>
+      <c r="G3043" s="0" t="inlineStr"/>
+      <c r="H3043" s="0" t="inlineStr"/>
     </row>
     <row r="3044">
-      <c r="A3044" t="inlineStr">
+      <c r="A3044" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3044" t="inlineStr">
+      <c r="B3044" s="0" t="inlineStr">
         <is>
           <t>装聋装哑</t>
         </is>
       </c>
-      <c r="C3044" t="inlineStr">
+      <c r="C3044" s="0" t="inlineStr">
         <is>
           <t>zhuānglóngzhuāngyǎ</t>
         </is>
       </c>
-      <c r="D3044" t="inlineStr">
+      <c r="D3044" s="0" t="inlineStr">
         <is>
           <t>假装听不见、说不出，故意不理</t>
         </is>
       </c>
-      <c r="E3044" t="inlineStr">
+      <c r="E3044" s="0" t="inlineStr">
         <is>
           <t>giả câm giả điếc</t>
         </is>
       </c>
-      <c r="F3044" t="inlineStr">
-        <is>
-          <t>有些人一谈到钱的问题就装聋装哑。</t>
-        </is>
-      </c>
-      <c r="G3044" t="inlineStr"/>
-      <c r="H3044" t="inlineStr"/>
+      <c r="F3044" s="0" t="inlineStr">
+        <is>
+          <t>同事之间闹矛盾的时候，我一般装聋装哑，不想卷进去。</t>
+        </is>
+      </c>
+      <c r="G3044" s="0" t="inlineStr"/>
+      <c r="H3044" s="0" t="inlineStr"/>
     </row>
     <row r="3045">
-      <c r="A3045" t="inlineStr">
+      <c r="A3045" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3045" t="inlineStr">
+      <c r="B3045" s="0" t="inlineStr">
         <is>
           <t>画蛇添足</t>
         </is>
       </c>
-      <c r="C3045" t="inlineStr">
+      <c r="C3045" s="0" t="inlineStr">
         <is>
           <t>huàshétiānzú</t>
         </is>
       </c>
-      <c r="D3045" t="inlineStr">
+      <c r="D3045" s="0" t="inlineStr">
         <is>
           <t>做多余的事，反而把事情弄坏</t>
         </is>
       </c>
-      <c r="E3045" t="inlineStr">
+      <c r="E3045" s="0" t="inlineStr">
         <is>
           <t>vẽ rắn thêm chân (làm thừa hỏng việc)</t>
         </is>
       </c>
-      <c r="F3045" t="inlineStr">
-        <is>
-          <t>这幅画已经很完美了，你就不要再画蛇添足了。</t>
-        </is>
-      </c>
-      <c r="G3045" t="inlineStr"/>
-      <c r="H3045" t="inlineStr"/>
+      <c r="F3045" s="0" t="inlineStr">
+        <is>
+          <t>这篇作文本来写得挺好，你再加那句反而画蛇添足了。</t>
+        </is>
+      </c>
+      <c r="G3045" s="0" t="inlineStr"/>
+      <c r="H3045" s="0" t="inlineStr"/>
     </row>
     <row r="3046">
-      <c r="A3046" t="inlineStr">
+      <c r="A3046" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3046" t="inlineStr">
+      <c r="B3046" s="0" t="inlineStr">
         <is>
           <t>机灵</t>
         </is>
       </c>
-      <c r="C3046" t="inlineStr">
+      <c r="C3046" s="0" t="inlineStr">
         <is>
           <t>jīling</t>
         </is>
       </c>
-      <c r="D3046" t="inlineStr">
+      <c r="D3046" s="0" t="inlineStr">
         <is>
           <t>聪明，反应很快</t>
         </is>
       </c>
-      <c r="E3046" t="inlineStr">
+      <c r="E3046" s="0" t="inlineStr">
         <is>
           <t>nhanh trí, lanh lợi</t>
         </is>
       </c>
-      <c r="F3046" t="inlineStr">
-        <is>
-          <t>小松鼠很机灵，听到一点动静就爬到树上去了。</t>
-        </is>
-      </c>
-      <c r="G3046" t="inlineStr"/>
-      <c r="H3046" t="inlineStr"/>
+      <c r="F3046" s="0" t="inlineStr">
+        <is>
+          <t>我班上有个学生特别机灵，一点就通。</t>
+        </is>
+      </c>
+      <c r="G3046" s="0" t="inlineStr"/>
+      <c r="H3046" s="0" t="inlineStr"/>
     </row>
     <row r="3047">
-      <c r="A3047" t="inlineStr">
+      <c r="A3047" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3047" t="inlineStr">
+      <c r="B3047" s="0" t="inlineStr">
         <is>
           <t>肆无忌惮</t>
         </is>
       </c>
-      <c r="C3047" t="inlineStr">
+      <c r="C3047" s="0" t="inlineStr">
         <is>
           <t>sìwújìdàn</t>
         </is>
       </c>
-      <c r="D3047" t="inlineStr">
+      <c r="D3047" s="0" t="inlineStr">
         <is>
           <t>一点也不怕、不顾忌，任意妄为</t>
         </is>
       </c>
-      <c r="E3047" t="inlineStr">
+      <c r="E3047" s="0" t="inlineStr">
         <is>
           <t>ngang nhiên, không kiêng nể gì</t>
         </is>
       </c>
-      <c r="F3047" t="inlineStr">
-        <is>
-          <t>对待坏人，我们越宽容，他们就越肆无忌惮。</t>
-        </is>
-      </c>
-      <c r="G3047" t="inlineStr"/>
-      <c r="H3047" t="inlineStr"/>
+      <c r="F3047" s="0" t="inlineStr">
+        <is>
+          <t>楼上的孩子晚上还肆无忌惮地跑来跑去，吵得我没法背书。</t>
+        </is>
+      </c>
+      <c r="G3047" s="0" t="inlineStr"/>
+      <c r="H3047" s="0" t="inlineStr"/>
     </row>
     <row r="3048">
-      <c r="A3048" t="inlineStr">
+      <c r="A3048" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3048" t="inlineStr">
+      <c r="B3048" s="0" t="inlineStr">
         <is>
           <t>损坏</t>
         </is>
       </c>
-      <c r="C3048" t="inlineStr">
+      <c r="C3048" s="0" t="inlineStr">
         <is>
           <t>sǔnhuài</t>
         </is>
       </c>
-      <c r="D3048" t="inlineStr">
+      <c r="D3048" s="0" t="inlineStr">
         <is>
           <t>使东西受到破坏、变坏</t>
         </is>
       </c>
-      <c r="E3048" t="inlineStr">
+      <c r="E3048" s="0" t="inlineStr">
         <is>
           <t>làm hỏng, hư hại</t>
         </is>
       </c>
-      <c r="F3048" t="inlineStr">
-        <is>
-          <t>机器需要经常维护，这样就不容易损坏。</t>
-        </is>
-      </c>
-      <c r="G3048" t="inlineStr"/>
-      <c r="H3048" t="inlineStr"/>
+      <c r="F3048" s="0" t="inlineStr">
+        <is>
+          <t>电脑突然损坏，我存的备考资料差点全丢了。</t>
+        </is>
+      </c>
+      <c r="G3048" s="0" t="inlineStr"/>
+      <c r="H3048" s="0" t="inlineStr"/>
     </row>
     <row r="3049">
-      <c r="A3049" t="inlineStr">
+      <c r="A3049" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3049" t="inlineStr">
+      <c r="B3049" s="0" t="inlineStr">
         <is>
           <t>倾向</t>
         </is>
       </c>
-      <c r="C3049" t="inlineStr">
+      <c r="C3049" s="0" t="inlineStr">
         <is>
           <t>qīngxiàng</t>
         </is>
       </c>
-      <c r="D3049" t="inlineStr">
+      <c r="D3049" s="0" t="inlineStr">
         <is>
           <t>更喜欢、更赞成某一方</t>
         </is>
       </c>
-      <c r="E3049" t="inlineStr">
+      <c r="E3049" s="0" t="inlineStr">
         <is>
           <t>nghiêng về, xu hướng</t>
         </is>
       </c>
-      <c r="F3049" t="inlineStr">
-        <is>
-          <t>虽然你们都不同意，但我更倾向于作者原意。</t>
-        </is>
-      </c>
-      <c r="G3049" t="inlineStr"/>
-      <c r="H3049" t="inlineStr"/>
+      <c r="F3049" s="0" t="inlineStr">
+        <is>
+          <t>选教材时，我更倾向于例句实用、贴近生活的那一套。</t>
+        </is>
+      </c>
+      <c r="G3049" s="0" t="inlineStr"/>
+      <c r="H3049" s="0" t="inlineStr"/>
     </row>
     <row r="3050">
-      <c r="A3050" t="inlineStr">
+      <c r="A3050" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3050" t="inlineStr">
+      <c r="B3050" s="0" t="inlineStr">
         <is>
           <t>试验</t>
         </is>
       </c>
-      <c r="C3050" t="inlineStr">
+      <c r="C3050" s="0" t="inlineStr">
         <is>
           <t>shìyàn</t>
         </is>
       </c>
-      <c r="D3050" t="inlineStr">
+      <c r="D3050" s="0" t="inlineStr">
         <is>
           <t>为了了解结果而进行的尝试</t>
         </is>
       </c>
-      <c r="E3050" t="inlineStr">
+      <c r="E3050" s="0" t="inlineStr">
         <is>
           <t>thử nghiệm</t>
         </is>
       </c>
-      <c r="F3050" t="inlineStr">
-        <is>
-          <t>那次试验因为准备不足，终于宣告失败。</t>
-        </is>
-      </c>
-      <c r="G3050" t="inlineStr"/>
-      <c r="H3050" t="inlineStr"/>
+      <c r="F3050" s="0" t="inlineStr">
+        <is>
+          <t>我打算试验一种新的背单词方法，看看效果怎么样。</t>
+        </is>
+      </c>
+      <c r="G3050" s="0" t="inlineStr"/>
+      <c r="H3050" s="0" t="inlineStr"/>
     </row>
     <row r="3051">
-      <c r="A3051" t="inlineStr">
+      <c r="A3051" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3051" t="inlineStr">
+      <c r="B3051" s="0" t="inlineStr">
         <is>
           <t>脂肪</t>
         </is>
       </c>
-      <c r="C3051" t="inlineStr">
+      <c r="C3051" s="0" t="inlineStr">
         <is>
           <t>zhīfáng</t>
         </is>
       </c>
-      <c r="D3051" t="inlineStr">
+      <c r="D3051" s="0" t="inlineStr">
         <is>
           <t>动物或人体内的油，肥肉部分</t>
         </is>
       </c>
-      <c r="E3051" t="inlineStr">
+      <c r="E3051" s="0" t="inlineStr">
         <is>
           <t>mỡ, chất béo</t>
         </is>
       </c>
-      <c r="F3051" t="inlineStr">
-        <is>
-          <t>冬天到了，别减肥了，留点儿脂肪抗寒。</t>
-        </is>
-      </c>
-      <c r="G3051" t="inlineStr"/>
-      <c r="H3051" t="inlineStr"/>
+      <c r="F3051" s="0" t="inlineStr">
+        <is>
+          <t>医生说我得多运动，少囤点脂肪。</t>
+        </is>
+      </c>
+      <c r="G3051" s="0" t="inlineStr"/>
+      <c r="H3051" s="0" t="inlineStr"/>
     </row>
     <row r="3052">
-      <c r="A3052" t="inlineStr">
+      <c r="A3052" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3052" t="inlineStr">
+      <c r="B3052" s="0" t="inlineStr">
         <is>
           <t>动脉</t>
         </is>
       </c>
-      <c r="C3052" t="inlineStr">
+      <c r="C3052" s="0" t="inlineStr">
         <is>
           <t>dòngmài</t>
         </is>
       </c>
-      <c r="D3052" t="inlineStr">
+      <c r="D3052" s="0" t="inlineStr">
         <is>
           <t>把血从心脏送到全身的血管</t>
         </is>
       </c>
-      <c r="E3052" t="inlineStr">
+      <c r="E3052" s="0" t="inlineStr">
         <is>
           <t>động mạch</t>
         </is>
       </c>
-      <c r="F3052" t="inlineStr">
-        <is>
-          <t>他激动得脖子旁边的大动脉都看得见跳动。</t>
-        </is>
-      </c>
-      <c r="G3052" t="inlineStr"/>
-      <c r="H3052" t="inlineStr"/>
+      <c r="F3052" s="0" t="inlineStr">
+        <is>
+          <t>我常跟学生说，语法就像句子的动脉，决定整句话通不通。</t>
+        </is>
+      </c>
+      <c r="G3052" s="0" t="inlineStr"/>
+      <c r="H3052" s="0" t="inlineStr"/>
     </row>
     <row r="3053">
-      <c r="A3053" t="inlineStr">
+      <c r="A3053" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3053" t="inlineStr">
+      <c r="B3053" s="0" t="inlineStr">
         <is>
           <t>实质</t>
         </is>
       </c>
-      <c r="C3053" t="inlineStr">
+      <c r="C3053" s="0" t="inlineStr">
         <is>
           <t>shízhì</t>
         </is>
       </c>
-      <c r="D3053" t="inlineStr">
+      <c r="D3053" s="0" t="inlineStr">
         <is>
           <t>事物真正的、本质的内容</t>
         </is>
       </c>
-      <c r="E3053" t="inlineStr">
+      <c r="E3053" s="0" t="inlineStr">
         <is>
           <t>thực chất, bản chất</t>
         </is>
       </c>
-      <c r="F3053" t="inlineStr">
-        <is>
-          <t>大家要认真领会文件的精神实质。</t>
-        </is>
-      </c>
-      <c r="G3053" t="inlineStr"/>
-      <c r="H3053" t="inlineStr"/>
+      <c r="F3053" s="0" t="inlineStr">
+        <is>
+          <t>学语言的实质不是背了多少词，而是能不能真正用出来。</t>
+        </is>
+      </c>
+      <c r="G3053" s="0" t="inlineStr"/>
+      <c r="H3053" s="0" t="inlineStr"/>
     </row>
     <row r="3054">
-      <c r="A3054" t="inlineStr">
+      <c r="A3054" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3054" t="inlineStr">
+      <c r="B3054" s="0" t="inlineStr">
         <is>
           <t>周密</t>
         </is>
       </c>
-      <c r="C3054" t="inlineStr">
+      <c r="C3054" s="0" t="inlineStr">
         <is>
           <t>zhōumì</t>
         </is>
       </c>
-      <c r="D3054" t="inlineStr">
+      <c r="D3054" s="0" t="inlineStr">
         <is>
           <t>考虑得很全面很细致，没有漏洞</t>
         </is>
       </c>
-      <c r="E3054" t="inlineStr">
+      <c r="E3054" s="0" t="inlineStr">
         <is>
           <t>chu đáo, kỹ lưỡng</t>
         </is>
       </c>
-      <c r="F3054" t="inlineStr">
-        <is>
-          <t>公安人员对这个案件做了周密的调查。</t>
-        </is>
-      </c>
-      <c r="G3054" t="inlineStr"/>
-      <c r="H3054" t="inlineStr"/>
+      <c r="F3054" s="0" t="inlineStr">
+        <is>
+          <t>考前我做了一个很周密的复习计划，每天学什么都排好了。</t>
+        </is>
+      </c>
+      <c r="G3054" s="0" t="inlineStr"/>
+      <c r="H3054" s="0" t="inlineStr"/>
     </row>
     <row r="3055">
-      <c r="A3055" t="inlineStr">
+      <c r="A3055" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3055" t="inlineStr">
+      <c r="B3055" s="0" t="inlineStr">
         <is>
           <t>途径</t>
         </is>
       </c>
-      <c r="C3055" t="inlineStr">
+      <c r="C3055" s="0" t="inlineStr">
         <is>
           <t>tújìng</t>
         </is>
       </c>
-      <c r="D3055" t="inlineStr">
+      <c r="D3055" s="0" t="inlineStr">
         <is>
           <t>达到目的的方法、门路</t>
         </is>
       </c>
-      <c r="E3055" t="inlineStr">
+      <c r="E3055" s="0" t="inlineStr">
         <is>
           <t>con đường, phương thức</t>
         </is>
       </c>
-      <c r="F3055" t="inlineStr">
-        <is>
-          <t>教育是提高国民素质的根本途径。</t>
-        </is>
-      </c>
-      <c r="G3055" t="inlineStr"/>
-      <c r="H3055" t="inlineStr"/>
+      <c r="F3055" s="0" t="inlineStr">
+        <is>
+          <t>多跟中国同事聊天，是我提高口语最有效的途径。</t>
+        </is>
+      </c>
+      <c r="G3055" s="0" t="inlineStr"/>
+      <c r="H3055" s="0" t="inlineStr"/>
     </row>
     <row r="3056">
-      <c r="A3056" t="inlineStr">
+      <c r="A3056" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3056" t="inlineStr">
+      <c r="B3056" s="0" t="inlineStr">
         <is>
           <t>虚假</t>
         </is>
       </c>
-      <c r="C3056" t="inlineStr">
+      <c r="C3056" s="0" t="inlineStr">
         <is>
           <t>xūjiǎ</t>
         </is>
       </c>
-      <c r="D3056" t="inlineStr">
+      <c r="D3056" s="0" t="inlineStr">
         <is>
           <t>不真实，假的</t>
         </is>
       </c>
-      <c r="E3056" t="inlineStr">
+      <c r="E3056" s="0" t="inlineStr">
         <is>
           <t>giả, không thật</t>
         </is>
       </c>
-      <c r="F3056" t="inlineStr">
-        <is>
-          <t>新闻报道必须真实，不许有半点虚假。</t>
-        </is>
-      </c>
-      <c r="G3056" t="inlineStr"/>
-      <c r="H3056" t="inlineStr"/>
+      <c r="F3056" s="0" t="inlineStr">
+        <is>
+          <t>网上很多“三个月过HSK6”的广告都很虚假。</t>
+        </is>
+      </c>
+      <c r="G3056" s="0" t="inlineStr"/>
+      <c r="H3056" s="0" t="inlineStr"/>
     </row>
     <row r="3057">
-      <c r="A3057" t="inlineStr">
+      <c r="A3057" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3057" t="inlineStr">
+      <c r="B3057" s="0" t="inlineStr">
         <is>
           <t>意向</t>
         </is>
       </c>
-      <c r="C3057" t="inlineStr">
+      <c r="C3057" s="0" t="inlineStr">
         <is>
           <t>yìxiàng</t>
         </is>
       </c>
-      <c r="D3057" t="inlineStr">
+      <c r="D3057" s="0" t="inlineStr">
         <is>
           <t>心里打算做某事的想法</t>
         </is>
       </c>
-      <c r="E3057" t="inlineStr">
+      <c r="E3057" s="0" t="inlineStr">
         <is>
           <t>ý định, ý hướng</t>
         </is>
       </c>
-      <c r="F3057" t="inlineStr">
-        <is>
-          <t>有多家企业表达了参与收购的意向。</t>
-        </is>
-      </c>
-      <c r="G3057" t="inlineStr"/>
-      <c r="H3057" t="inlineStr"/>
+      <c r="F3057" s="0" t="inlineStr">
+        <is>
+          <t>我跟中心表达了想多带几节口语课的意向。</t>
+        </is>
+      </c>
+      <c r="G3057" s="0" t="inlineStr"/>
+      <c r="H3057" s="0" t="inlineStr"/>
     </row>
     <row r="3058">
-      <c r="A3058" t="inlineStr">
+      <c r="A3058" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3058" t="inlineStr">
+      <c r="B3058" s="0" t="inlineStr">
         <is>
           <t>一丝不苟</t>
         </is>
       </c>
-      <c r="C3058" t="inlineStr">
+      <c r="C3058" s="0" t="inlineStr">
         <is>
           <t>yìsībùgǒu</t>
         </is>
       </c>
-      <c r="D3058" t="inlineStr">
+      <c r="D3058" s="0" t="inlineStr">
         <is>
           <t>做事非常认真，一点也不马虎</t>
         </is>
       </c>
-      <c r="E3058" t="inlineStr">
+      <c r="E3058" s="0" t="inlineStr">
         <is>
           <t>tỉ mỉ, không cẩu thả chút nào</t>
         </is>
       </c>
-      <c r="F3058" t="inlineStr">
-        <is>
-          <t>张老师对待教学工作一向严肃认真，一丝不苟。</t>
-        </is>
-      </c>
-      <c r="G3058" t="inlineStr"/>
-      <c r="H3058" t="inlineStr"/>
+      <c r="F3058" s="0" t="inlineStr">
+        <is>
+          <t>批改学生作业时，我总是一丝不苟，连一个标点都不放过。</t>
+        </is>
+      </c>
+      <c r="G3058" s="0" t="inlineStr"/>
+      <c r="H3058" s="0" t="inlineStr"/>
     </row>
     <row r="3059">
-      <c r="A3059" t="inlineStr">
+      <c r="A3059" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3059" t="inlineStr">
+      <c r="B3059" s="0" t="inlineStr">
         <is>
           <t>收益</t>
         </is>
       </c>
-      <c r="C3059" t="inlineStr">
+      <c r="C3059" s="0" t="inlineStr">
         <is>
           <t>shōuyì</t>
         </is>
       </c>
-      <c r="D3059" t="inlineStr">
+      <c r="D3059" s="0" t="inlineStr">
         <is>
           <t>得到的好处或利润</t>
         </is>
       </c>
-      <c r="E3059" t="inlineStr">
+      <c r="E3059" s="0" t="inlineStr">
         <is>
           <t>lợi ích/lợi nhuận thu về</t>
         </is>
       </c>
-      <c r="F3059" t="inlineStr">
-        <is>
-          <t>理财产品的收益越大，风险就越高。</t>
-        </is>
-      </c>
-      <c r="G3059" t="inlineStr"/>
-      <c r="H3059" t="inlineStr"/>
+      <c r="F3059" s="0" t="inlineStr">
+        <is>
+          <t>每天坚持学两小时，时间一长，收益特别明显。</t>
+        </is>
+      </c>
+      <c r="G3059" s="0" t="inlineStr"/>
+      <c r="H3059" s="0" t="inlineStr"/>
     </row>
     <row r="3060">
-      <c r="A3060" t="inlineStr">
+      <c r="A3060" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3060" t="inlineStr">
+      <c r="B3060" s="0" t="inlineStr">
         <is>
           <t>恰当</t>
         </is>
       </c>
-      <c r="C3060" t="inlineStr">
+      <c r="C3060" s="0" t="inlineStr">
         <is>
           <t>qiàdàng</t>
         </is>
       </c>
-      <c r="D3060" t="inlineStr">
+      <c r="D3060" s="0" t="inlineStr">
         <is>
           <t>正合适，不多不少</t>
         </is>
       </c>
-      <c r="E3060" t="inlineStr">
+      <c r="E3060" s="0" t="inlineStr">
         <is>
           <t>thích đáng, thỏa đáng</t>
         </is>
       </c>
-      <c r="F3060" t="inlineStr">
-        <is>
-          <t>恰当地使用形容词，可以使文章更加生动。</t>
-        </is>
-      </c>
-      <c r="G3060" t="inlineStr"/>
-      <c r="H3060" t="inlineStr"/>
+      <c r="F3060" s="0" t="inlineStr">
+        <is>
+          <t>用词是否恰当，往往决定一篇HSK作文的分数。</t>
+        </is>
+      </c>
+      <c r="G3060" s="0" t="inlineStr"/>
+      <c r="H3060" s="0" t="inlineStr"/>
     </row>
     <row r="3061">
-      <c r="A3061" t="inlineStr">
+      <c r="A3061" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3061" t="inlineStr">
+      <c r="B3061" s="0" t="inlineStr">
         <is>
           <t>特定</t>
         </is>
       </c>
-      <c r="C3061" t="inlineStr">
+      <c r="C3061" s="0" t="inlineStr">
         <is>
           <t>tèdìng</t>
         </is>
       </c>
-      <c r="D3061" t="inlineStr">
+      <c r="D3061" s="0" t="inlineStr">
         <is>
           <t>特别指定的，某一个固定的</t>
         </is>
       </c>
-      <c r="E3061" t="inlineStr">
+      <c r="E3061" s="0" t="inlineStr">
         <is>
           <t>đặc định, nhất định</t>
         </is>
       </c>
-      <c r="F3061" t="inlineStr">
-        <is>
-          <t>在那特定的生活环境里养成了她孤僻的性格。</t>
-        </is>
-      </c>
-      <c r="G3061" t="inlineStr"/>
-      <c r="H3061" t="inlineStr"/>
+      <c r="F3061" s="0" t="inlineStr">
+        <is>
+          <t>有些词只在特定场合才用，用错了会显得很奇怪。</t>
+        </is>
+      </c>
+      <c r="G3061" s="0" t="inlineStr"/>
+      <c r="H3061" s="0" t="inlineStr"/>
     </row>
     <row r="3062">
-      <c r="A3062" t="inlineStr">
+      <c r="A3062" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3062" t="inlineStr">
+      <c r="B3062" s="0" t="inlineStr">
         <is>
           <t>缘故</t>
         </is>
       </c>
-      <c r="C3062" t="inlineStr">
+      <c r="C3062" s="0" t="inlineStr">
         <is>
           <t>yuángù</t>
         </is>
       </c>
-      <c r="D3062" t="inlineStr">
+      <c r="D3062" s="0" t="inlineStr">
         <is>
           <t>原因</t>
         </is>
       </c>
-      <c r="E3062" t="inlineStr">
+      <c r="E3062" s="0" t="inlineStr">
         <is>
           <t>nguyên cớ, lý do</t>
         </is>
       </c>
-      <c r="F3062" t="inlineStr">
-        <is>
-          <t>由于雷雨的缘故，飞机起飞的时间再次变更了。</t>
-        </is>
-      </c>
-      <c r="G3062" t="inlineStr"/>
-      <c r="H3062" t="inlineStr"/>
+      <c r="F3062" s="0" t="inlineStr">
+        <is>
+          <t>不知什么缘故，这几个生词我怎么背都记不住。</t>
+        </is>
+      </c>
+      <c r="G3062" s="0" t="inlineStr"/>
+      <c r="H3062" s="0" t="inlineStr"/>
     </row>
     <row r="3063">
-      <c r="A3063" t="inlineStr">
+      <c r="A3063" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3063" t="inlineStr">
+      <c r="B3063" s="0" t="inlineStr">
         <is>
           <t>诚挚</t>
         </is>
       </c>
-      <c r="C3063" t="inlineStr">
+      <c r="C3063" s="0" t="inlineStr">
         <is>
           <t>chéngzhì</t>
         </is>
       </c>
-      <c r="D3063" t="inlineStr">
+      <c r="D3063" s="0" t="inlineStr">
         <is>
           <t>真诚而恳切</t>
         </is>
       </c>
-      <c r="E3063" t="inlineStr">
+      <c r="E3063" s="0" t="inlineStr">
         <is>
           <t>chân thành, thành khẩn</t>
         </is>
       </c>
-      <c r="F3063" t="inlineStr">
-        <is>
-          <t>会谈是在诚挚友好的气氛中进行的。</t>
-        </is>
-      </c>
-      <c r="G3063" t="inlineStr"/>
-      <c r="H3063" t="inlineStr"/>
+      <c r="F3063" s="0" t="inlineStr">
+        <is>
+          <t>学生毕业时给我写了一段很诚挚的话，我特别感动。</t>
+        </is>
+      </c>
+      <c r="G3063" s="0" t="inlineStr"/>
+      <c r="H3063" s="0" t="inlineStr"/>
     </row>
     <row r="3064">
-      <c r="A3064" t="inlineStr">
+      <c r="A3064" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3064" t="inlineStr">
+      <c r="B3064" s="0" t="inlineStr">
         <is>
           <t>倾听</t>
         </is>
       </c>
-      <c r="C3064" t="inlineStr">
+      <c r="C3064" s="0" t="inlineStr">
         <is>
           <t>qīngtīng</t>
         </is>
       </c>
-      <c r="D3064" t="inlineStr">
+      <c r="D3064" s="0" t="inlineStr">
         <is>
           <t>认真、用心地听别人说</t>
         </is>
       </c>
-      <c r="E3064" t="inlineStr">
+      <c r="E3064" s="0" t="inlineStr">
         <is>
           <t>lắng nghe</t>
         </is>
       </c>
-      <c r="F3064" t="inlineStr">
-        <is>
-          <t>了解别人最好的方式就是倾听。</t>
-        </is>
-      </c>
-      <c r="G3064" t="inlineStr"/>
-      <c r="H3064" t="inlineStr"/>
+      <c r="F3064" s="0" t="inlineStr">
+        <is>
+          <t>教低年级的孩子，耐心倾听有时比急着纠错更重要。</t>
+        </is>
+      </c>
+      <c r="G3064" s="0" t="inlineStr"/>
+      <c r="H3064" s="0" t="inlineStr"/>
     </row>
     <row r="3065">
-      <c r="A3065" t="inlineStr">
+      <c r="A3065" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3065" t="inlineStr">
+      <c r="B3065" s="0" t="inlineStr">
         <is>
           <t>视频</t>
         </is>
       </c>
-      <c r="C3065" t="inlineStr">
+      <c r="C3065" s="0" t="inlineStr">
         <is>
           <t>shìpín</t>
         </is>
       </c>
-      <c r="D3065" t="inlineStr">
+      <c r="D3065" s="0" t="inlineStr">
         <is>
           <t>能看到画面的影像</t>
         </is>
       </c>
-      <c r="E3065" t="inlineStr">
+      <c r="E3065" s="0" t="inlineStr">
         <is>
           <t>video, đoạn phim</t>
         </is>
       </c>
-      <c r="F3065" t="inlineStr">
-        <is>
-          <t>看了关于长江黄河的视频，我真想亲眼去看看。</t>
-        </is>
-      </c>
-      <c r="G3065" t="inlineStr"/>
-      <c r="H3065" t="inlineStr"/>
+      <c r="F3065" s="0" t="inlineStr">
+        <is>
+          <t>每天早上我都会看一段中文视频来练听力。</t>
+        </is>
+      </c>
+      <c r="G3065" s="0" t="inlineStr"/>
+      <c r="H3065" s="0" t="inlineStr"/>
     </row>
     <row r="3066">
-      <c r="A3066" t="inlineStr">
+      <c r="A3066" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3066" t="inlineStr">
+      <c r="B3066" s="0" t="inlineStr">
         <is>
           <t>一目了然</t>
         </is>
       </c>
-      <c r="C3066" t="inlineStr">
+      <c r="C3066" s="0" t="inlineStr">
         <is>
           <t>yímùliǎorán</t>
         </is>
       </c>
-      <c r="D3066" t="inlineStr">
+      <c r="D3066" s="0" t="inlineStr">
         <is>
           <t>一眼就能看清楚</t>
         </is>
       </c>
-      <c r="E3066" t="inlineStr">
+      <c r="E3066" s="0" t="inlineStr">
         <is>
           <t>nhìn là hiểu ngay, rõ mồn một</t>
         </is>
       </c>
-      <c r="F3066" t="inlineStr">
-        <is>
-          <t>陈列室明亮宽敞，展品一目了然。</t>
-        </is>
-      </c>
-      <c r="G3066" t="inlineStr"/>
-      <c r="H3066" t="inlineStr"/>
+      <c r="F3066" s="0" t="inlineStr">
+        <is>
+          <t>我把语法做成表格，学生一看就一目了然。</t>
+        </is>
+      </c>
+      <c r="G3066" s="0" t="inlineStr"/>
+      <c r="H3066" s="0" t="inlineStr"/>
     </row>
     <row r="3067">
-      <c r="A3067" t="inlineStr">
+      <c r="A3067" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3067" t="inlineStr">
+      <c r="B3067" s="0" t="inlineStr">
         <is>
           <t>提炼</t>
         </is>
       </c>
-      <c r="C3067" t="inlineStr">
+      <c r="C3067" s="0" t="inlineStr">
         <is>
           <t>tíliàn</t>
         </is>
       </c>
-      <c r="D3067" t="inlineStr">
+      <c r="D3067" s="0" t="inlineStr">
         <is>
           <t>从原料里提取有用的东西；使更精纯</t>
         </is>
       </c>
-      <c r="E3067" t="inlineStr">
+      <c r="E3067" s="0" t="inlineStr">
         <is>
           <t>chiết luyện, chắt lọc</t>
         </is>
       </c>
-      <c r="F3067" t="inlineStr">
-        <is>
-          <t>橄榄可提炼出珍贵的橄榄油。</t>
-        </is>
-      </c>
-      <c r="G3067" t="inlineStr"/>
-      <c r="H3067" t="inlineStr"/>
+      <c r="F3067" s="0" t="inlineStr">
+        <is>
+          <t>读完一篇文章，我会试着把重点提炼成几句话。</t>
+        </is>
+      </c>
+      <c r="G3067" s="0" t="inlineStr"/>
+      <c r="H3067" s="0" t="inlineStr"/>
     </row>
     <row r="3068">
-      <c r="A3068" t="inlineStr">
+      <c r="A3068" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3068" t="inlineStr">
+      <c r="B3068" s="0" t="inlineStr">
         <is>
           <t>探测</t>
         </is>
       </c>
-      <c r="C3068" t="inlineStr">
+      <c r="C3068" s="0" t="inlineStr">
         <is>
           <t>tàncè</t>
         </is>
       </c>
-      <c r="D3068" t="inlineStr">
+      <c r="D3068" s="0" t="inlineStr">
         <is>
           <t>用仪器去测量、察看看不见的东西</t>
         </is>
       </c>
-      <c r="E3068" t="inlineStr">
+      <c r="E3068" s="0" t="inlineStr">
         <is>
           <t>thăm dò, dò tìm</t>
         </is>
       </c>
-      <c r="F3068" t="inlineStr">
-        <is>
-          <t>这些军用犬可以帮助我们探测到爆炸物。</t>
-        </is>
-      </c>
-      <c r="G3068" t="inlineStr"/>
-      <c r="H3068" t="inlineStr"/>
+      <c r="F3068" s="0" t="inlineStr">
+        <is>
+          <t>上课前我常先探测一下学生已经掌握到什么程度。</t>
+        </is>
+      </c>
+      <c r="G3068" s="0" t="inlineStr"/>
+      <c r="H3068" s="0" t="inlineStr"/>
     </row>
     <row r="3069">
-      <c r="A3069" t="inlineStr">
+      <c r="A3069" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3069" t="inlineStr">
+      <c r="B3069" s="0" t="inlineStr">
         <is>
           <t>智商</t>
         </is>
       </c>
-      <c r="C3069" t="inlineStr">
+      <c r="C3069" s="0" t="inlineStr">
         <is>
           <t>zhìshāng</t>
         </is>
       </c>
-      <c r="D3069" t="inlineStr">
+      <c r="D3069" s="0" t="inlineStr">
         <is>
           <t>衡量聪明程度的指数（IQ）</t>
         </is>
       </c>
-      <c r="E3069" t="inlineStr">
+      <c r="E3069" s="0" t="inlineStr">
         <is>
           <t>chỉ số thông minh (IQ)</t>
         </is>
       </c>
-      <c r="F3069" t="inlineStr">
-        <is>
-          <t>智商就是我们常说的IQ。</t>
-        </is>
-      </c>
-      <c r="G3069" t="inlineStr"/>
-      <c r="H3069" t="inlineStr"/>
+      <c r="F3069" s="0" t="inlineStr">
+        <is>
+          <t>学好一门语言靠的不是高智商，而是每天的坚持。</t>
+        </is>
+      </c>
+      <c r="G3069" s="0" t="inlineStr"/>
+      <c r="H3069" s="0" t="inlineStr"/>
     </row>
     <row r="3070">
-      <c r="A3070" t="inlineStr">
+      <c r="A3070" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3070" t="inlineStr">
+      <c r="B3070" s="0" t="inlineStr">
         <is>
           <t>探讨</t>
         </is>
       </c>
-      <c r="C3070" t="inlineStr">
+      <c r="C3070" s="0" t="inlineStr">
         <is>
           <t>tàntǎo</t>
         </is>
       </c>
-      <c r="D3070" t="inlineStr">
+      <c r="D3070" s="0" t="inlineStr">
         <is>
           <t>一起研究、讨论问题</t>
         </is>
       </c>
-      <c r="E3070" t="inlineStr">
+      <c r="E3070" s="0" t="inlineStr">
         <is>
           <t>thảo luận, tìm tòi</t>
         </is>
       </c>
-      <c r="F3070" t="inlineStr">
-        <is>
-          <t>专家们一起探讨治理污水的问题。</t>
-        </is>
-      </c>
-      <c r="G3070" t="inlineStr"/>
-      <c r="H3070" t="inlineStr"/>
+      <c r="F3070" s="0" t="inlineStr">
+        <is>
+          <t>我常跟同事一起探讨怎么把课上得更有意思。</t>
+        </is>
+      </c>
+      <c r="G3070" s="0" t="inlineStr"/>
+      <c r="H3070" s="0" t="inlineStr"/>
     </row>
     <row r="3071">
-      <c r="A3071" t="inlineStr">
+      <c r="A3071" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3071" t="inlineStr">
+      <c r="B3071" s="0" t="inlineStr">
         <is>
           <t>分寸</t>
         </is>
       </c>
-      <c r="C3071" t="inlineStr">
+      <c r="C3071" s="0" t="inlineStr">
         <is>
           <t>fēncun</t>
         </is>
       </c>
-      <c r="D3071" t="inlineStr">
+      <c r="D3071" s="0" t="inlineStr">
         <is>
           <t>说话做事的适当程度、界限</t>
         </is>
       </c>
-      <c r="E3071" t="inlineStr">
+      <c r="E3071" s="0" t="inlineStr">
         <is>
           <t>chừng mực, mức độ phải chăng</t>
         </is>
       </c>
-      <c r="F3071" t="inlineStr">
-        <is>
-          <t>我们说话、做事都要掌握适当的分寸。</t>
-        </is>
-      </c>
-      <c r="G3071" t="inlineStr"/>
-      <c r="H3071" t="inlineStr"/>
+      <c r="F3071" s="0" t="inlineStr">
+        <is>
+          <t>纠正学生发音的时候也要讲分寸，不能太打击他们。</t>
+        </is>
+      </c>
+      <c r="G3071" s="0" t="inlineStr"/>
+      <c r="H3071" s="0" t="inlineStr"/>
     </row>
     <row r="3072">
-      <c r="A3072" t="inlineStr">
+      <c r="A3072" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3072" t="inlineStr">
+      <c r="B3072" s="0" t="inlineStr">
         <is>
           <t>恰到好处</t>
         </is>
       </c>
-      <c r="C3072" t="inlineStr">
+      <c r="C3072" s="0" t="inlineStr">
         <is>
           <t>qiàdàohǎochù</t>
         </is>
       </c>
-      <c r="D3072" t="inlineStr">
+      <c r="D3072" s="0" t="inlineStr">
         <is>
           <t>正好达到最合适的程度</t>
         </is>
       </c>
-      <c r="E3072" t="inlineStr">
+      <c r="E3072" s="0" t="inlineStr">
         <is>
           <t>vừa vặn, đúng mức</t>
         </is>
       </c>
-      <c r="F3072" t="inlineStr">
-        <is>
-          <t>他用适当的方法，恰到好处地处理了这件事。</t>
-        </is>
-      </c>
-      <c r="G3072" t="inlineStr"/>
-      <c r="H3072" t="inlineStr"/>
+      <c r="F3072" s="0" t="inlineStr">
+        <is>
+          <t>好老师提问的难度总是恰到好处，不会太难也不会太简单。</t>
+        </is>
+      </c>
+      <c r="G3072" s="0" t="inlineStr"/>
+      <c r="H3072" s="0" t="inlineStr"/>
     </row>
     <row r="3073">
-      <c r="A3073" t="inlineStr">
+      <c r="A3073" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3073" t="inlineStr">
+      <c r="B3073" s="0" t="inlineStr">
         <is>
           <t>是非</t>
         </is>
       </c>
-      <c r="C3073" t="inlineStr">
+      <c r="C3073" s="0" t="inlineStr">
         <is>
           <t>shìfēi</t>
         </is>
       </c>
-      <c r="D3073" t="inlineStr">
+      <c r="D3073" s="0" t="inlineStr">
         <is>
           <t>对和错</t>
         </is>
       </c>
-      <c r="E3073" t="inlineStr">
+      <c r="E3073" s="0" t="inlineStr">
         <is>
           <t>thị phi, đúng sai</t>
         </is>
       </c>
-      <c r="F3073" t="inlineStr">
-        <is>
-          <t>我们要努力提高分辨是非的能力。</t>
-        </is>
-      </c>
-      <c r="G3073" t="inlineStr"/>
-      <c r="H3073" t="inlineStr"/>
+      <c r="F3073" s="0" t="inlineStr">
+        <is>
+          <t>办公室里的那些是非我一向不参与，专心做自己的事。</t>
+        </is>
+      </c>
+      <c r="G3073" s="0" t="inlineStr"/>
+      <c r="H3073" s="0" t="inlineStr"/>
     </row>
     <row r="3074">
-      <c r="A3074" t="inlineStr">
+      <c r="A3074" s="0" t="inlineStr">
         <is>
           <t>Bài 29</t>
         </is>
       </c>
-      <c r="B3074" t="inlineStr">
+      <c r="B3074" s="0" t="inlineStr">
         <is>
           <t>起哄</t>
         </is>
       </c>
-      <c r="C3074" t="inlineStr">
+      <c r="C3074" s="0" t="inlineStr">
         <is>
           <t>qǐhòng</t>
         </is>
       </c>
-      <c r="D3074" t="inlineStr">
+      <c r="D3074" s="0" t="inlineStr">
         <is>
           <t>很多人一起吵闹、捣乱</t>
         </is>
       </c>
-      <c r="E3074" t="inlineStr">
+      <c r="E3074" s="0" t="inlineStr">
         <is>
           <t>hùa theo làm ầm ĩ, la ó</t>
         </is>
       </c>
-      <c r="F3074" t="inlineStr">
-        <is>
-          <t>小明没有弄清情况，就跟着人家瞎起哄。</t>
-        </is>
-      </c>
-      <c r="G3074" t="inlineStr"/>
-      <c r="H3074" t="inlineStr"/>
+      <c r="F3074" s="0" t="inlineStr">
+        <is>
+          <t>学生一起哄，课堂纪律一下子就乱了。</t>
+        </is>
+      </c>
+      <c r="G3074" s="0" t="inlineStr"/>
+      <c r="H3074" s="0" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H1:H3025">

</xml_diff>

<commit_message>
feat(vocab-study): nghĩa Việt + 例句 cá nhân hoá HSK6 + sửa bug drop dòng
- vi_override.json: 1167 nghĩa Việt (Bài 1-28) lấp cột 意义 trống; build_md fallback, Excel ưu tiên
- ex_override.json: 621 例句 cá nhân hoá (Bài 15-28) bám user-profile; GHI ĐÈ câu bài khóa
- render_html: sửa bug bỏ nhầm dòng dữ liệu có "---" trong ô (khôi phục 勉强 Bài 5)
- SKILL.md: tài liệu hoá 2 override mới + luật hàng phân cách bảng
- Ra soat: 生词 1422 | Nghĩa Việt trống 0 | override -> html 1167/1167 + 621/621 (đồng bộ)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/raw/Từ vựng.xlsx
+++ b/raw/Từ vựng.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB3074"/>
+  <dimension ref="A1:AB3124"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="13.13" customWidth="1" style="24" min="1" max="1"/>
@@ -72671,6 +72671,1706 @@
       </c>
       <c r="G3074" s="0" t="inlineStr"/>
       <c r="H3074" s="0" t="inlineStr"/>
+    </row>
+    <row r="3075">
+      <c r="A3075" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3075" t="inlineStr">
+        <is>
+          <t>容忍</t>
+        </is>
+      </c>
+      <c r="C3075" t="inlineStr">
+        <is>
+          <t>róngrěn</t>
+        </is>
+      </c>
+      <c r="D3075" t="inlineStr">
+        <is>
+          <t>宽容忍耐，不计较别人的过错</t>
+        </is>
+      </c>
+      <c r="E3075" t="inlineStr">
+        <is>
+          <t>dung thứ, khoan dung</t>
+        </is>
+      </c>
+      <c r="F3075" t="inlineStr">
+        <is>
+          <t>备考HSK6压力大，我尽量容忍自己偶尔想偷懒的心情。</t>
+        </is>
+      </c>
+      <c r="G3075" t="inlineStr"/>
+      <c r="H3075" t="inlineStr"/>
+    </row>
+    <row r="3076">
+      <c r="A3076" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3076" t="inlineStr">
+        <is>
+          <t>蹬</t>
+        </is>
+      </c>
+      <c r="C3076" t="inlineStr">
+        <is>
+          <t>dēng</t>
+        </is>
+      </c>
+      <c r="D3076" t="inlineStr">
+        <is>
+          <t>用脚用力踩或踏</t>
+        </is>
+      </c>
+      <c r="E3076" t="inlineStr">
+        <is>
+          <t>đạp (chân)</t>
+        </is>
+      </c>
+      <c r="F3076" t="inlineStr">
+        <is>
+          <t>每天下班我都骑共享单车回家，上坡时得使劲蹬。</t>
+        </is>
+      </c>
+      <c r="G3076" t="inlineStr"/>
+      <c r="H3076" t="inlineStr"/>
+    </row>
+    <row r="3077">
+      <c r="A3077" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3077" t="inlineStr">
+        <is>
+          <t>拳头</t>
+        </is>
+      </c>
+      <c r="C3077" t="inlineStr">
+        <is>
+          <t>quántou</t>
+        </is>
+      </c>
+      <c r="D3077" t="inlineStr">
+        <is>
+          <t>手指弯曲合拢握紧的手</t>
+        </is>
+      </c>
+      <c r="E3077" t="inlineStr">
+        <is>
+          <t>nắm đấm</t>
+        </is>
+      </c>
+      <c r="F3077" t="inlineStr">
+        <is>
+          <t>教HSK1的“手”字时，我握起拳头给小朋友做示范。</t>
+        </is>
+      </c>
+      <c r="G3077" t="inlineStr"/>
+      <c r="H3077" t="inlineStr"/>
+    </row>
+    <row r="3078">
+      <c r="A3078" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3078" t="inlineStr">
+        <is>
+          <t>不时</t>
+        </is>
+      </c>
+      <c r="C3078" t="inlineStr">
+        <is>
+          <t>bùshí</t>
+        </is>
+      </c>
+      <c r="D3078" t="inlineStr">
+        <is>
+          <t>时常，一次又一次地（多用于书面）</t>
+        </is>
+      </c>
+      <c r="E3078" t="inlineStr">
+        <is>
+          <t>thường xuyên, chốc chốc lại</t>
+        </is>
+      </c>
+      <c r="F3078" t="inlineStr">
+        <is>
+          <t>上中文课时，学生不时举手提问，我很喜欢这种气氛。</t>
+        </is>
+      </c>
+      <c r="G3078" t="inlineStr"/>
+      <c r="H3078" t="inlineStr"/>
+    </row>
+    <row r="3079">
+      <c r="A3079" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3079" t="inlineStr">
+        <is>
+          <t>气色</t>
+        </is>
+      </c>
+      <c r="C3079" t="inlineStr">
+        <is>
+          <t>qìsè</t>
+        </is>
+      </c>
+      <c r="D3079" t="inlineStr">
+        <is>
+          <t>人脸上表现出来的健康状况</t>
+        </is>
+      </c>
+      <c r="E3079" t="inlineStr">
+        <is>
+          <t>sắc mặt, thần sắc</t>
+        </is>
+      </c>
+      <c r="F3079" t="inlineStr">
+        <is>
+          <t>昨晚熬夜背单词，今天同事说我气色不太好。</t>
+        </is>
+      </c>
+      <c r="G3079" t="inlineStr"/>
+      <c r="H3079" t="inlineStr"/>
+    </row>
+    <row r="3080">
+      <c r="A3080" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3080" t="inlineStr">
+        <is>
+          <t>轨道</t>
+        </is>
+      </c>
+      <c r="C3080" t="inlineStr">
+        <is>
+          <t>guǐdào</t>
+        </is>
+      </c>
+      <c r="D3080" t="inlineStr">
+        <is>
+          <t>火车、地铁行驶的路线；也比喻正常发展的路子</t>
+        </is>
+      </c>
+      <c r="E3080" t="inlineStr">
+        <is>
+          <t>đường ray; quỹ đạo</t>
+        </is>
+      </c>
+      <c r="F3080" t="inlineStr">
+        <is>
+          <t>备考计划乱了一阵，现在又回到了正常轨道。</t>
+        </is>
+      </c>
+      <c r="G3080" t="inlineStr"/>
+      <c r="H3080" t="inlineStr"/>
+    </row>
+    <row r="3081">
+      <c r="A3081" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3081" t="inlineStr">
+        <is>
+          <t>酒精</t>
+        </is>
+      </c>
+      <c r="C3081" t="inlineStr">
+        <is>
+          <t>jiǔjīng</t>
+        </is>
+      </c>
+      <c r="D3081" t="inlineStr">
+        <is>
+          <t>酒里能使人醉的成分</t>
+        </is>
+      </c>
+      <c r="E3081" t="inlineStr">
+        <is>
+          <t>cồn, chất cồn (trong rượu)</t>
+        </is>
+      </c>
+      <c r="F3081" t="inlineStr">
+        <is>
+          <t>在中国跟同事聚餐时，我一般不喝酒精含量高的白酒。</t>
+        </is>
+      </c>
+      <c r="G3081" t="inlineStr"/>
+      <c r="H3081" t="inlineStr"/>
+    </row>
+    <row r="3082">
+      <c r="A3082" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3082" t="inlineStr">
+        <is>
+          <t>竭尽全力</t>
+        </is>
+      </c>
+      <c r="C3082" t="inlineStr">
+        <is>
+          <t>jiéjìn quánlì</t>
+        </is>
+      </c>
+      <c r="D3082" t="inlineStr">
+        <is>
+          <t>用尽全部的力量</t>
+        </is>
+      </c>
+      <c r="E3082" t="inlineStr">
+        <is>
+          <t>dốc hết sức, gắng hết sức</t>
+        </is>
+      </c>
+      <c r="F3082" t="inlineStr">
+        <is>
+          <t>为了HSKK拿高分，我竭尽全力每天练口语。</t>
+        </is>
+      </c>
+      <c r="G3082" t="inlineStr"/>
+      <c r="H3082" t="inlineStr"/>
+    </row>
+    <row r="3083">
+      <c r="A3083" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3083" t="inlineStr">
+        <is>
+          <t>根源</t>
+        </is>
+      </c>
+      <c r="C3083" t="inlineStr">
+        <is>
+          <t>gēnyuán</t>
+        </is>
+      </c>
+      <c r="D3083" t="inlineStr">
+        <is>
+          <t>事情产生的根本原因</t>
+        </is>
+      </c>
+      <c r="E3083" t="inlineStr">
+        <is>
+          <t>nguồn gốc, căn nguyên</t>
+        </is>
+      </c>
+      <c r="F3083" t="inlineStr">
+        <is>
+          <t>我发现自己听力差的根源是平时听得太少。</t>
+        </is>
+      </c>
+      <c r="G3083" t="inlineStr"/>
+      <c r="H3083" t="inlineStr"/>
+    </row>
+    <row r="3084">
+      <c r="A3084" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3084" t="inlineStr">
+        <is>
+          <t>对付</t>
+        </is>
+      </c>
+      <c r="C3084" t="inlineStr">
+        <is>
+          <t>duìfu</t>
+        </is>
+      </c>
+      <c r="D3084" t="inlineStr">
+        <is>
+          <t>想办法处理人或事情</t>
+        </is>
+      </c>
+      <c r="E3084" t="inlineStr">
+        <is>
+          <t>đối phó, ứng phó</t>
+        </is>
+      </c>
+      <c r="F3084" t="inlineStr">
+        <is>
+          <t>遇到不会做的HSK6阅读题，我有一套自己对付的办法。</t>
+        </is>
+      </c>
+      <c r="G3084" t="inlineStr"/>
+      <c r="H3084" t="inlineStr"/>
+    </row>
+    <row r="3085">
+      <c r="A3085" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3085" t="inlineStr">
+        <is>
+          <t>纠正</t>
+        </is>
+      </c>
+      <c r="C3085" t="inlineStr">
+        <is>
+          <t>jiūzhèng</t>
+        </is>
+      </c>
+      <c r="D3085" t="inlineStr">
+        <is>
+          <t>改正错误</t>
+        </is>
+      </c>
+      <c r="E3085" t="inlineStr">
+        <is>
+          <t>sửa chữa, uốn nắn</t>
+        </is>
+      </c>
+      <c r="F3085" t="inlineStr">
+        <is>
+          <t>上课时我会及时纠正学生的发音错误。</t>
+        </is>
+      </c>
+      <c r="G3085" t="inlineStr"/>
+      <c r="H3085" t="inlineStr"/>
+    </row>
+    <row r="3086">
+      <c r="A3086" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3086" t="inlineStr">
+        <is>
+          <t>糟蹋</t>
+        </is>
+      </c>
+      <c r="C3086" t="inlineStr">
+        <is>
+          <t>zāotà</t>
+        </is>
+      </c>
+      <c r="D3086" t="inlineStr">
+        <is>
+          <t>浪费或随意损坏（东西、身体等）</t>
+        </is>
+      </c>
+      <c r="E3086" t="inlineStr">
+        <is>
+          <t>phí phạm, tàn phá</t>
+        </is>
+      </c>
+      <c r="F3086" t="inlineStr">
+        <is>
+          <t>经常熬夜其实就是在糟蹋自己的身体。</t>
+        </is>
+      </c>
+      <c r="G3086" t="inlineStr"/>
+      <c r="H3086" t="inlineStr"/>
+    </row>
+    <row r="3087">
+      <c r="A3087" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3087" t="inlineStr">
+        <is>
+          <t>迫害</t>
+        </is>
+      </c>
+      <c r="C3087" t="inlineStr">
+        <is>
+          <t>pòhài</t>
+        </is>
+      </c>
+      <c r="D3087" t="inlineStr">
+        <is>
+          <t>用暴力或权势残酷地压迫、伤害</t>
+        </is>
+      </c>
+      <c r="E3087" t="inlineStr">
+        <is>
+          <t>bức hại</t>
+        </is>
+      </c>
+      <c r="F3087" t="inlineStr">
+        <is>
+          <t>这部纪录片讲的是战争年代很多人遭到迫害的故事。</t>
+        </is>
+      </c>
+      <c r="G3087" t="inlineStr"/>
+      <c r="H3087" t="inlineStr"/>
+    </row>
+    <row r="3088">
+      <c r="A3088" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3088" t="inlineStr">
+        <is>
+          <t>毁灭</t>
+        </is>
+      </c>
+      <c r="C3088" t="inlineStr">
+        <is>
+          <t>huǐmiè</t>
+        </is>
+      </c>
+      <c r="D3088" t="inlineStr">
+        <is>
+          <t>彻底摧毁，使不再存在</t>
+        </is>
+      </c>
+      <c r="E3088" t="inlineStr">
+        <is>
+          <t>hủy diệt, phá hủy</t>
+        </is>
+      </c>
+      <c r="F3088" t="inlineStr">
+        <is>
+          <t>坏习惯会一点一点毁灭一个人的健康。</t>
+        </is>
+      </c>
+      <c r="G3088" t="inlineStr"/>
+      <c r="H3088" t="inlineStr"/>
+    </row>
+    <row r="3089">
+      <c r="A3089" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3089" t="inlineStr">
+        <is>
+          <t>惯例</t>
+        </is>
+      </c>
+      <c r="C3089" t="inlineStr">
+        <is>
+          <t>guànlì</t>
+        </is>
+      </c>
+      <c r="D3089" t="inlineStr">
+        <is>
+          <t>一向的做法，习惯上的规矩</t>
+        </is>
+      </c>
+      <c r="E3089" t="inlineStr">
+        <is>
+          <t>thông lệ, lệ thường</t>
+        </is>
+      </c>
+      <c r="F3089" t="inlineStr">
+        <is>
+          <t>按照惯例，我每天早上先复习昨天学的生词。</t>
+        </is>
+      </c>
+      <c r="G3089" t="inlineStr"/>
+      <c r="H3089" t="inlineStr"/>
+    </row>
+    <row r="3090">
+      <c r="A3090" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3090" t="inlineStr">
+        <is>
+          <t>顽固</t>
+        </is>
+      </c>
+      <c r="C3090" t="inlineStr">
+        <is>
+          <t>wángù</t>
+        </is>
+      </c>
+      <c r="D3090" t="inlineStr">
+        <is>
+          <t>思想保守、不肯改变；（病）难治</t>
+        </is>
+      </c>
+      <c r="E3090" t="inlineStr">
+        <is>
+          <t>ngoan cố; dai dẳng (bệnh)</t>
+        </is>
+      </c>
+      <c r="F3090" t="inlineStr">
+        <is>
+          <t>我有个顽固的坏习惯，就是睡前老爱看手机。</t>
+        </is>
+      </c>
+      <c r="G3090" t="inlineStr"/>
+      <c r="H3090" t="inlineStr"/>
+    </row>
+    <row r="3091">
+      <c r="A3091" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3091" t="inlineStr">
+        <is>
+          <t>奢侈</t>
+        </is>
+      </c>
+      <c r="C3091" t="inlineStr">
+        <is>
+          <t>shēchǐ</t>
+        </is>
+      </c>
+      <c r="D3091" t="inlineStr">
+        <is>
+          <t>花很多钱财追求享受</t>
+        </is>
+      </c>
+      <c r="E3091" t="inlineStr">
+        <is>
+          <t>xa xỉ, xa hoa</t>
+        </is>
+      </c>
+      <c r="F3091" t="inlineStr">
+        <is>
+          <t>对上班族来说，能睡到自然醒简直是一种奢侈。</t>
+        </is>
+      </c>
+      <c r="G3091" t="inlineStr"/>
+      <c r="H3091" t="inlineStr"/>
+    </row>
+    <row r="3092">
+      <c r="A3092" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3092" t="inlineStr">
+        <is>
+          <t>指数</t>
+        </is>
+      </c>
+      <c r="C3092" t="inlineStr">
+        <is>
+          <t>zhǐshù</t>
+        </is>
+      </c>
+      <c r="D3092" t="inlineStr">
+        <is>
+          <t>用来表示某种情况变动的数值</t>
+        </is>
+      </c>
+      <c r="E3092" t="inlineStr">
+        <is>
+          <t>chỉ số</t>
+        </is>
+      </c>
+      <c r="F3092" t="inlineStr">
+        <is>
+          <t>中国发布的睡眠指数显示很多人睡眠质量不高。</t>
+        </is>
+      </c>
+      <c r="G3092" t="inlineStr"/>
+      <c r="H3092" t="inlineStr"/>
+    </row>
+    <row r="3093">
+      <c r="A3093" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3093" t="inlineStr">
+        <is>
+          <t>居民</t>
+        </is>
+      </c>
+      <c r="C3093" t="inlineStr">
+        <is>
+          <t>jūmín</t>
+        </is>
+      </c>
+      <c r="D3093" t="inlineStr">
+        <is>
+          <t>住在某个地方的人</t>
+        </is>
+      </c>
+      <c r="E3093" t="inlineStr">
+        <is>
+          <t>cư dân, dân cư</t>
+        </is>
+      </c>
+      <c r="F3093" t="inlineStr">
+        <is>
+          <t>我住的小区居民大多是年轻上班族。</t>
+        </is>
+      </c>
+      <c r="G3093" t="inlineStr"/>
+      <c r="H3093" t="inlineStr"/>
+    </row>
+    <row r="3094">
+      <c r="A3094" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3094" t="inlineStr">
+        <is>
+          <t>当前</t>
+        </is>
+      </c>
+      <c r="C3094" t="inlineStr">
+        <is>
+          <t>dāngqián</t>
+        </is>
+      </c>
+      <c r="D3094" t="inlineStr">
+        <is>
+          <t>目前，现在这个时候</t>
+        </is>
+      </c>
+      <c r="E3094" t="inlineStr">
+        <is>
+          <t>hiện nay, trước mắt</t>
+        </is>
+      </c>
+      <c r="F3094" t="inlineStr">
+        <is>
+          <t>当前我最重要的任务就是顺利通过HSK6。</t>
+        </is>
+      </c>
+      <c r="G3094" t="inlineStr"/>
+      <c r="H3094" t="inlineStr"/>
+    </row>
+    <row r="3095">
+      <c r="A3095" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3095" t="inlineStr">
+        <is>
+          <t>扰乱</t>
+        </is>
+      </c>
+      <c r="C3095" t="inlineStr">
+        <is>
+          <t>rǎoluàn</t>
+        </is>
+      </c>
+      <c r="D3095" t="inlineStr">
+        <is>
+          <t>打乱，使变得混乱</t>
+        </is>
+      </c>
+      <c r="E3095" t="inlineStr">
+        <is>
+          <t>quấy nhiễu, làm rối loạn</t>
+        </is>
+      </c>
+      <c r="F3095" t="inlineStr">
+        <is>
+          <t>睡前刷手机会扰乱我的作息。</t>
+        </is>
+      </c>
+      <c r="G3095" t="inlineStr"/>
+      <c r="H3095" t="inlineStr"/>
+    </row>
+    <row r="3096">
+      <c r="A3096" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3096" t="inlineStr">
+        <is>
+          <t>折腾</t>
+        </is>
+      </c>
+      <c r="C3096" t="inlineStr">
+        <is>
+          <t>zhēteng</t>
+        </is>
+      </c>
+      <c r="D3096" t="inlineStr">
+        <is>
+          <t>反复做某事；使身心不得安宁</t>
+        </is>
+      </c>
+      <c r="E3096" t="inlineStr">
+        <is>
+          <t>hành hạ; trằn trọc, quần quật</t>
+        </is>
+      </c>
+      <c r="F3096" t="inlineStr">
+        <is>
+          <t>昨晚失眠，我在床上翻来覆去折腾了大半夜。</t>
+        </is>
+      </c>
+      <c r="G3096" t="inlineStr"/>
+      <c r="H3096" t="inlineStr"/>
+    </row>
+    <row r="3097">
+      <c r="A3097" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3097" t="inlineStr">
+        <is>
+          <t>逆行</t>
+        </is>
+      </c>
+      <c r="C3097" t="inlineStr">
+        <is>
+          <t>nìxíng</t>
+        </is>
+      </c>
+      <c r="D3097" t="inlineStr">
+        <is>
+          <t>朝着跟规定相反的方向行进</t>
+        </is>
+      </c>
+      <c r="E3097" t="inlineStr">
+        <is>
+          <t>đi ngược chiều</t>
+        </is>
+      </c>
+      <c r="F3097" t="inlineStr">
+        <is>
+          <t>在中国骑车千万不能逆行，太危险了。</t>
+        </is>
+      </c>
+      <c r="G3097" t="inlineStr"/>
+      <c r="H3097" t="inlineStr"/>
+    </row>
+    <row r="3098">
+      <c r="A3098" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3098" t="inlineStr">
+        <is>
+          <t>茫然</t>
+        </is>
+      </c>
+      <c r="C3098" t="inlineStr">
+        <is>
+          <t>mángrán</t>
+        </is>
+      </c>
+      <c r="D3098" t="inlineStr">
+        <is>
+          <t>完全不知道，心里没有主意的样子</t>
+        </is>
+      </c>
+      <c r="E3098" t="inlineStr">
+        <is>
+          <t>mờ mịt, ngơ ngác</t>
+        </is>
+      </c>
+      <c r="F3098" t="inlineStr">
+        <is>
+          <t>刚开始学HSK6语法时，我常常一脸茫然。</t>
+        </is>
+      </c>
+      <c r="G3098" t="inlineStr"/>
+      <c r="H3098" t="inlineStr"/>
+    </row>
+    <row r="3099">
+      <c r="A3099" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3099" t="inlineStr">
+        <is>
+          <t>丢三落四</t>
+        </is>
+      </c>
+      <c r="C3099" t="inlineStr">
+        <is>
+          <t>diūsān-làsì</t>
+        </is>
+      </c>
+      <c r="D3099" t="inlineStr">
+        <is>
+          <t>做事马虎，常常有遗漏</t>
+        </is>
+      </c>
+      <c r="E3099" t="inlineStr">
+        <is>
+          <t>đầu quên đuôi, hay quên</t>
+        </is>
+      </c>
+      <c r="F3099" t="inlineStr">
+        <is>
+          <t>我记性不好，出门总是丢三落四。</t>
+        </is>
+      </c>
+      <c r="G3099" t="inlineStr"/>
+      <c r="H3099" t="inlineStr"/>
+    </row>
+    <row r="3100">
+      <c r="A3100" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3100" t="inlineStr">
+        <is>
+          <t>起伏</t>
+        </is>
+      </c>
+      <c r="C3100" t="inlineStr">
+        <is>
+          <t>qǐfú</t>
+        </is>
+      </c>
+      <c r="D3100" t="inlineStr">
+        <is>
+          <t>一起一落；（情绪等）变化不定</t>
+        </is>
+      </c>
+      <c r="E3100" t="inlineStr">
+        <is>
+          <t>nhấp nhô; thăng trầm, biến động</t>
+        </is>
+      </c>
+      <c r="F3100" t="inlineStr">
+        <is>
+          <t>备考那段时间我情绪起伏很大，一会儿信心满满，一会儿又想放弃。</t>
+        </is>
+      </c>
+      <c r="G3100" t="inlineStr"/>
+      <c r="H3100" t="inlineStr"/>
+    </row>
+    <row r="3101">
+      <c r="A3101" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3101" t="inlineStr">
+        <is>
+          <t>发呆</t>
+        </is>
+      </c>
+      <c r="C3101" t="inlineStr">
+        <is>
+          <t>fādāi</t>
+        </is>
+      </c>
+      <c r="D3101" t="inlineStr">
+        <is>
+          <t>因为出神而呆呆地不动</t>
+        </is>
+      </c>
+      <c r="E3101" t="inlineStr">
+        <is>
+          <t>thẫn thờ, ngẩn người ra</t>
+        </is>
+      </c>
+      <c r="F3101" t="inlineStr">
+        <is>
+          <t>单词背累了，我常常对着窗外发呆。</t>
+        </is>
+      </c>
+      <c r="G3101" t="inlineStr"/>
+      <c r="H3101" t="inlineStr"/>
+    </row>
+    <row r="3102">
+      <c r="A3102" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3102" t="inlineStr">
+        <is>
+          <t>记性</t>
+        </is>
+      </c>
+      <c r="C3102" t="inlineStr">
+        <is>
+          <t>jìxing</t>
+        </is>
+      </c>
+      <c r="D3102" t="inlineStr">
+        <is>
+          <t>记忆的能力</t>
+        </is>
+      </c>
+      <c r="E3102" t="inlineStr">
+        <is>
+          <t>trí nhớ</t>
+        </is>
+      </c>
+      <c r="F3102" t="inlineStr">
+        <is>
+          <t>睡不好觉，我的记性明显变差了。</t>
+        </is>
+      </c>
+      <c r="G3102" t="inlineStr"/>
+      <c r="H3102" t="inlineStr"/>
+    </row>
+    <row r="3103">
+      <c r="A3103" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3103" t="inlineStr">
+        <is>
+          <t>摧残</t>
+        </is>
+      </c>
+      <c r="C3103" t="inlineStr">
+        <is>
+          <t>cuīcán</t>
+        </is>
+      </c>
+      <c r="D3103" t="inlineStr">
+        <is>
+          <t>使受到严重的损害</t>
+        </is>
+      </c>
+      <c r="E3103" t="inlineStr">
+        <is>
+          <t>tàn phá, dày vò</t>
+        </is>
+      </c>
+      <c r="F3103" t="inlineStr">
+        <is>
+          <t>长期熬夜会摧残身体健康。</t>
+        </is>
+      </c>
+      <c r="G3103" t="inlineStr"/>
+      <c r="H3103" t="inlineStr"/>
+    </row>
+    <row r="3104">
+      <c r="A3104" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3104" t="inlineStr">
+        <is>
+          <t>普及</t>
+        </is>
+      </c>
+      <c r="C3104" t="inlineStr">
+        <is>
+          <t>pǔjí</t>
+        </is>
+      </c>
+      <c r="D3104" t="inlineStr">
+        <is>
+          <t>普遍推广，使大家都有或都懂</t>
+        </is>
+      </c>
+      <c r="E3104" t="inlineStr">
+        <is>
+          <t>phổ cập, phổ biến</t>
+        </is>
+      </c>
+      <c r="F3104" t="inlineStr">
+        <is>
+          <t>智能手机普及以后，很多人睡前都离不开它。</t>
+        </is>
+      </c>
+      <c r="G3104" t="inlineStr"/>
+      <c r="H3104" t="inlineStr"/>
+    </row>
+    <row r="3105">
+      <c r="A3105" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3105" t="inlineStr">
+        <is>
+          <t>盛行</t>
+        </is>
+      </c>
+      <c r="C3105" t="inlineStr">
+        <is>
+          <t>shèngxíng</t>
+        </is>
+      </c>
+      <c r="D3105" t="inlineStr">
+        <is>
+          <t>广泛地流行</t>
+        </is>
+      </c>
+      <c r="E3105" t="inlineStr">
+        <is>
+          <t>thịnh hành, phổ biến rộng</t>
+        </is>
+      </c>
+      <c r="F3105" t="inlineStr">
+        <is>
+          <t>现在睡前上网的习惯很盛行。</t>
+        </is>
+      </c>
+      <c r="G3105" t="inlineStr"/>
+      <c r="H3105" t="inlineStr"/>
+    </row>
+    <row r="3106">
+      <c r="A3106" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3106" t="inlineStr">
+        <is>
+          <t>细胞</t>
+        </is>
+      </c>
+      <c r="C3106" t="inlineStr">
+        <is>
+          <t>xìbāo</t>
+        </is>
+      </c>
+      <c r="D3106" t="inlineStr">
+        <is>
+          <t>生物体结构和功能的基本单位</t>
+        </is>
+      </c>
+      <c r="E3106" t="inlineStr">
+        <is>
+          <t>tế bào</t>
+        </is>
+      </c>
+      <c r="F3106" t="inlineStr">
+        <is>
+          <t>熬夜会影响人体细胞的正常活动。</t>
+        </is>
+      </c>
+      <c r="G3106" t="inlineStr"/>
+      <c r="H3106" t="inlineStr"/>
+    </row>
+    <row r="3107">
+      <c r="A3107" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3107" t="inlineStr">
+        <is>
+          <t>肿瘤</t>
+        </is>
+      </c>
+      <c r="C3107" t="inlineStr">
+        <is>
+          <t>zhǒngliú</t>
+        </is>
+      </c>
+      <c r="D3107" t="inlineStr">
+        <is>
+          <t>身体里不正常增生的组织块</t>
+        </is>
+      </c>
+      <c r="E3107" t="inlineStr">
+        <is>
+          <t>khối u, u bướu</t>
+        </is>
+      </c>
+      <c r="F3107" t="inlineStr">
+        <is>
+          <t>医生说定期体检能早点发现肿瘤。</t>
+        </is>
+      </c>
+      <c r="G3107" t="inlineStr"/>
+      <c r="H3107" t="inlineStr"/>
+    </row>
+    <row r="3108">
+      <c r="A3108" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3108" t="inlineStr">
+        <is>
+          <t>癌症</t>
+        </is>
+      </c>
+      <c r="C3108" t="inlineStr">
+        <is>
+          <t>áizhèng</t>
+        </is>
+      </c>
+      <c r="D3108" t="inlineStr">
+        <is>
+          <t>由恶性肿瘤引起的疾病</t>
+        </is>
+      </c>
+      <c r="E3108" t="inlineStr">
+        <is>
+          <t>bệnh ung thư</t>
+        </is>
+      </c>
+      <c r="F3108" t="inlineStr">
+        <is>
+          <t>不良的生活习惯可能会增加得癌症的风险。</t>
+        </is>
+      </c>
+      <c r="G3108" t="inlineStr"/>
+      <c r="H3108" t="inlineStr"/>
+    </row>
+    <row r="3109">
+      <c r="A3109" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3109" t="inlineStr">
+        <is>
+          <t>呼吁</t>
+        </is>
+      </c>
+      <c r="C3109" t="inlineStr">
+        <is>
+          <t>hūyù</t>
+        </is>
+      </c>
+      <c r="D3109" t="inlineStr">
+        <is>
+          <t>大声向社会请求支持或帮助</t>
+        </is>
+      </c>
+      <c r="E3109" t="inlineStr">
+        <is>
+          <t>kêu gọi</t>
+        </is>
+      </c>
+      <c r="F3109" t="inlineStr">
+        <is>
+          <t>医生呼吁大家不要经常熬夜。</t>
+        </is>
+      </c>
+      <c r="G3109" t="inlineStr"/>
+      <c r="H3109" t="inlineStr"/>
+    </row>
+    <row r="3110">
+      <c r="A3110" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3110" t="inlineStr">
+        <is>
+          <t>无动于衷</t>
+        </is>
+      </c>
+      <c r="C3110" t="inlineStr">
+        <is>
+          <t>wúdòngyúzhōng</t>
+        </is>
+      </c>
+      <c r="D3110" t="inlineStr">
+        <is>
+          <t>心里一点儿也不受触动，毫不在意</t>
+        </is>
+      </c>
+      <c r="E3110" t="inlineStr">
+        <is>
+          <t>thờ ơ, dửng dưng</t>
+        </is>
+      </c>
+      <c r="F3110" t="inlineStr">
+        <is>
+          <t>对自己的坏习惯不能无动于衷，要及时改正。</t>
+        </is>
+      </c>
+      <c r="G3110" t="inlineStr"/>
+      <c r="H3110" t="inlineStr"/>
+    </row>
+    <row r="3111">
+      <c r="A3111" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3111" t="inlineStr">
+        <is>
+          <t>过瘾</t>
+        </is>
+      </c>
+      <c r="C3111" t="inlineStr">
+        <is>
+          <t>guòyǐn</t>
+        </is>
+      </c>
+      <c r="D3111" t="inlineStr">
+        <is>
+          <t>满足了某种爱好，觉得很痛快</t>
+        </is>
+      </c>
+      <c r="E3111" t="inlineStr">
+        <is>
+          <t>đã, thỏa mãn (sở thích)</t>
+        </is>
+      </c>
+      <c r="F3111" t="inlineStr">
+        <is>
+          <t>周末追一整天中文剧，看得特别过瘾。</t>
+        </is>
+      </c>
+      <c r="G3111" t="inlineStr"/>
+      <c r="H3111" t="inlineStr"/>
+    </row>
+    <row r="3112">
+      <c r="A3112" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3112" t="inlineStr">
+        <is>
+          <t>分泌</t>
+        </is>
+      </c>
+      <c r="C3112" t="inlineStr">
+        <is>
+          <t>fēnmì</t>
+        </is>
+      </c>
+      <c r="D3112" t="inlineStr">
+        <is>
+          <t>生物体产生并排出某种物质</t>
+        </is>
+      </c>
+      <c r="E3112" t="inlineStr">
+        <is>
+          <t>tiết ra, bài tiết</t>
+        </is>
+      </c>
+      <c r="F3112" t="inlineStr">
+        <is>
+          <t>光污染会影响人体褪黑素的分泌。</t>
+        </is>
+      </c>
+      <c r="G3112" t="inlineStr"/>
+      <c r="H3112" t="inlineStr"/>
+    </row>
+    <row r="3113">
+      <c r="A3113" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3113" t="inlineStr">
+        <is>
+          <t>职能</t>
+        </is>
+      </c>
+      <c r="C3113" t="inlineStr">
+        <is>
+          <t>zhínéng</t>
+        </is>
+      </c>
+      <c r="D3113" t="inlineStr">
+        <is>
+          <t>事物或机构应有的功能、作用</t>
+        </is>
+      </c>
+      <c r="E3113" t="inlineStr">
+        <is>
+          <t>chức năng</t>
+        </is>
+      </c>
+      <c r="F3113" t="inlineStr">
+        <is>
+          <t>褪黑素的一个重要职能是帮助睡眠。</t>
+        </is>
+      </c>
+      <c r="G3113" t="inlineStr"/>
+      <c r="H3113" t="inlineStr"/>
+    </row>
+    <row r="3114">
+      <c r="A3114" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3114" t="inlineStr">
+        <is>
+          <t>衰老</t>
+        </is>
+      </c>
+      <c r="C3114" t="inlineStr">
+        <is>
+          <t>shuāilǎo</t>
+        </is>
+      </c>
+      <c r="D3114" t="inlineStr">
+        <is>
+          <t>身体机能因年老而衰退</t>
+        </is>
+      </c>
+      <c r="E3114" t="inlineStr">
+        <is>
+          <t>già đi, lão hóa</t>
+        </is>
+      </c>
+      <c r="F3114" t="inlineStr">
+        <is>
+          <t>睡眠不足会让人加速衰老。</t>
+        </is>
+      </c>
+      <c r="G3114" t="inlineStr"/>
+      <c r="H3114" t="inlineStr"/>
+    </row>
+    <row r="3115">
+      <c r="A3115" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3115" t="inlineStr">
+        <is>
+          <t>调剂</t>
+        </is>
+      </c>
+      <c r="C3115" t="inlineStr">
+        <is>
+          <t>tiáojì</t>
+        </is>
+      </c>
+      <c r="D3115" t="inlineStr">
+        <is>
+          <t>调整使合适；调节</t>
+        </is>
+      </c>
+      <c r="E3115" t="inlineStr">
+        <is>
+          <t>điều tiết, điều hòa</t>
+        </is>
+      </c>
+      <c r="F3115" t="inlineStr">
+        <is>
+          <t>学习累了，我会听听音乐调剂一下心情。</t>
+        </is>
+      </c>
+      <c r="G3115" t="inlineStr"/>
+      <c r="H3115" t="inlineStr"/>
+    </row>
+    <row r="3116">
+      <c r="A3116" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3116" t="inlineStr">
+        <is>
+          <t>供不应求</t>
+        </is>
+      </c>
+      <c r="C3116" t="inlineStr">
+        <is>
+          <t>gōngbùyìngqiú</t>
+        </is>
+      </c>
+      <c r="D3116" t="inlineStr">
+        <is>
+          <t>供应满足不了需求</t>
+        </is>
+      </c>
+      <c r="E3116" t="inlineStr">
+        <is>
+          <t>cung không đủ cầu</t>
+        </is>
+      </c>
+      <c r="F3116" t="inlineStr">
+        <is>
+          <t>在中国，好的睡眠门诊医生总是供不应求。</t>
+        </is>
+      </c>
+      <c r="G3116" t="inlineStr"/>
+      <c r="H3116" t="inlineStr"/>
+    </row>
+    <row r="3117">
+      <c r="A3117" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3117" t="inlineStr">
+        <is>
+          <t>不相上下</t>
+        </is>
+      </c>
+      <c r="C3117" t="inlineStr">
+        <is>
+          <t>bùxiāng-shàngxià</t>
+        </is>
+      </c>
+      <c r="D3117" t="inlineStr">
+        <is>
+          <t>分不出高低好坏，程度差不多</t>
+        </is>
+      </c>
+      <c r="E3117" t="inlineStr">
+        <is>
+          <t>ngang tài ngang sức, xấp xỉ</t>
+        </is>
+      </c>
+      <c r="F3117" t="inlineStr">
+        <is>
+          <t>我和同桌的汉语水平不相上下。</t>
+        </is>
+      </c>
+      <c r="G3117" t="inlineStr"/>
+      <c r="H3117" t="inlineStr"/>
+    </row>
+    <row r="3118">
+      <c r="A3118" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3118" t="inlineStr">
+        <is>
+          <t>总而言之</t>
+        </is>
+      </c>
+      <c r="C3118" t="inlineStr">
+        <is>
+          <t>zǒng'éryánzhī</t>
+        </is>
+      </c>
+      <c r="D3118" t="inlineStr">
+        <is>
+          <t>总的说来</t>
+        </is>
+      </c>
+      <c r="E3118" t="inlineStr">
+        <is>
+          <t>tóm lại, nói tóm lại</t>
+        </is>
+      </c>
+      <c r="F3118" t="inlineStr">
+        <is>
+          <t>总而言之，想学好中文，坚持最重要。</t>
+        </is>
+      </c>
+      <c r="G3118" t="inlineStr"/>
+      <c r="H3118" t="inlineStr"/>
+    </row>
+    <row r="3119">
+      <c r="A3119" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3119" t="inlineStr">
+        <is>
+          <t>恶化</t>
+        </is>
+      </c>
+      <c r="C3119" t="inlineStr">
+        <is>
+          <t>èhuà</t>
+        </is>
+      </c>
+      <c r="D3119" t="inlineStr">
+        <is>
+          <t>情况向坏的方向发展</t>
+        </is>
+      </c>
+      <c r="E3119" t="inlineStr">
+        <is>
+          <t>xấu đi, trở nặng</t>
+        </is>
+      </c>
+      <c r="F3119" t="inlineStr">
+        <is>
+          <t>如果一直睡不好，健康状况会慢慢恶化。</t>
+        </is>
+      </c>
+      <c r="G3119" t="inlineStr"/>
+      <c r="H3119" t="inlineStr"/>
+    </row>
+    <row r="3120">
+      <c r="A3120" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3120" t="inlineStr">
+        <is>
+          <t>适宜</t>
+        </is>
+      </c>
+      <c r="C3120" t="inlineStr">
+        <is>
+          <t>shìyí</t>
+        </is>
+      </c>
+      <c r="D3120" t="inlineStr">
+        <is>
+          <t>合适，恰当</t>
+        </is>
+      </c>
+      <c r="E3120" t="inlineStr">
+        <is>
+          <t>thích hợp, phù hợp</t>
+        </is>
+      </c>
+      <c r="F3120" t="inlineStr">
+        <is>
+          <t>睡前听点轻音乐，很适宜放松心情。</t>
+        </is>
+      </c>
+      <c r="G3120" t="inlineStr"/>
+      <c r="H3120" t="inlineStr"/>
+    </row>
+    <row r="3121">
+      <c r="A3121" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3121" t="inlineStr">
+        <is>
+          <t>场合</t>
+        </is>
+      </c>
+      <c r="C3121" t="inlineStr">
+        <is>
+          <t>chǎnghé</t>
+        </is>
+      </c>
+      <c r="D3121" t="inlineStr">
+        <is>
+          <t>一定的时间、地点和情况</t>
+        </is>
+      </c>
+      <c r="E3121" t="inlineStr">
+        <is>
+          <t>trường hợp, dịp, hoàn cảnh</t>
+        </is>
+      </c>
+      <c r="F3121" t="inlineStr">
+        <is>
+          <t>在正式场合，我说中文会更客气一些。</t>
+        </is>
+      </c>
+      <c r="G3121" t="inlineStr"/>
+      <c r="H3121" t="inlineStr"/>
+    </row>
+    <row r="3122">
+      <c r="A3122" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3122" t="inlineStr">
+        <is>
+          <t>地步</t>
+        </is>
+      </c>
+      <c r="C3122" t="inlineStr">
+        <is>
+          <t>dìbù</t>
+        </is>
+      </c>
+      <c r="D3122" t="inlineStr">
+        <is>
+          <t>达到的程度（多指不好的情况）</t>
+        </is>
+      </c>
+      <c r="E3122" t="inlineStr">
+        <is>
+          <t>mức độ, nước (đến nước)</t>
+        </is>
+      </c>
+      <c r="F3122" t="inlineStr">
+        <is>
+          <t>那阵子我忙到连饭都顾不上吃的地步。</t>
+        </is>
+      </c>
+      <c r="G3122" t="inlineStr"/>
+      <c r="H3122" t="inlineStr"/>
+    </row>
+    <row r="3123">
+      <c r="A3123" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3123" t="inlineStr">
+        <is>
+          <t>混乱</t>
+        </is>
+      </c>
+      <c r="C3123" t="inlineStr">
+        <is>
+          <t>hùnluàn</t>
+        </is>
+      </c>
+      <c r="D3123" t="inlineStr">
+        <is>
+          <t>没有条理，乱七八糟</t>
+        </is>
+      </c>
+      <c r="E3123" t="inlineStr">
+        <is>
+          <t>hỗn loạn, lộn xộn</t>
+        </is>
+      </c>
+      <c r="F3123" t="inlineStr">
+        <is>
+          <t>睡不好觉时，我的思路会变得很混乱。</t>
+        </is>
+      </c>
+      <c r="G3123" t="inlineStr"/>
+      <c r="H3123" t="inlineStr"/>
+    </row>
+    <row r="3124">
+      <c r="A3124" t="inlineStr">
+        <is>
+          <t>Bài 30</t>
+        </is>
+      </c>
+      <c r="B3124" t="inlineStr">
+        <is>
+          <t>举足轻重</t>
+        </is>
+      </c>
+      <c r="C3124" t="inlineStr">
+        <is>
+          <t>jǔzú-qīngzhòng</t>
+        </is>
+      </c>
+      <c r="D3124" t="inlineStr">
+        <is>
+          <t>所处地位重要，一举一动都影响全局</t>
+        </is>
+      </c>
+      <c r="E3124" t="inlineStr">
+        <is>
+          <t>có vai trò then chốt, cực kỳ quan trọng</t>
+        </is>
+      </c>
+      <c r="F3124" t="inlineStr">
+        <is>
+          <t>睡眠对健康举足轻重，千万不能忽视。</t>
+        </is>
+      </c>
+      <c r="G3124" t="inlineStr"/>
+      <c r="H3124" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H1:H3025">

</xml_diff>